<commit_message>
Alpha7 step 13: ONE BAR content, conductor balance, three bug fixes
- 6 motifs (DOWNBEAT, ENTRANCE, GREEN ROOM, UNISON, SEGUE, LAST WORD)
- 4 enemies (ROOM TONE, THE CUE, THE DAMPER, STUTTER) and elite THE ROUND
- 3 events (A RIVAL BAND, A TUNING FORK, A CRACKED BOW)
- band damage to enemies goes through Strike, move strength through MoveScale
- conductors closer together: FUGUE x1.8, DUET 12/8, THE SUN 8, CAPRICE 20 percent
- fixes: enemy intent on a fallen musician, 7th bench chip under PLAY THE BAR,
  BAR TOTAL missing the bar's last turn
- turnsim saves BREATH for a CALL and takes TACET_SIM_SEED; turncheck 109/109

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WqLsaY7gVTeQY89VfVgASG
</commit_message>
<xml_diff>
--- a/docs/TACET_Balance.xlsx
+++ b/docs/TACET_Balance.xlsx
@@ -1470,7 +1470,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A54"/>
+  <dimension ref="A1:A59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="140" customWidth="1" style="33" min="1" max="1"/>
@@ -1508,105 +1508,105 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t xml:space="preserve">  FLAWLESS  FLOOR 1  EARLY 100%  2.0b   0% 2.0c   LATE  100%  3.0b   0% 2.0c   ELITE 100%  3.0b   0% 1.9c   BOSS  100%  4.9b   0% 2.0c   </t>
+          <t xml:space="preserve">  FLAWLESS  FLOOR 1  EARLY 100%  2.0b   0% 1.8c   LATE  100%  2.9b   0% 2.0c   ELITE 100%  3.0b   0% 1.9c   BOSS  100%  4.9b   0% 2.0c   </t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t xml:space="preserve">  FLAWLESS  FLOOR 2  EARLY 100%  3.0b   0% 2.0c   LATE  100%  3.1b   0% 2.0c   ELITE 100%  4.0b   0% 2.0c   BOSS  100%  5.7b   0% 2.0c   </t>
+          <t xml:space="preserve">  FLAWLESS  FLOOR 2  EARLY 100%  3.0b   0% 2.0c   LATE  100%  3.2b   0% 2.0c   ELITE 100%  3.9b   0% 2.0c   BOSS  100%  5.7b   0% 2.0c   </t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t xml:space="preserve">  FLAWLESS  FLOOR 3  EARLY 100%  4.0b   0% 2.0c   LATE  100%  4.0b   0% 2.0c   ELITE 100%  4.5b   0% 2.0c   BOSS  100%  6.8b   0% 2.0c   </t>
+          <t xml:space="preserve">  FLAWLESS  FLOOR 3  EARLY 100%  3.9b   0% 2.0c   LATE  100%  4.2b   0% 2.0c   ELITE 100%  4.4b   0% 2.0c   BOSS  100%  6.9b   0% 2.0c   </t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t xml:space="preserve">  EXPERT    FLOOR 1  EARLY 100%  2.0b   2% 1.6c   LATE  100%  3.0b   5% 2.0c   ELITE 100%  3.3b   6% 1.9c   BOSS  100%  5.2b  12% 1.9c   </t>
+          <t xml:space="preserve">  EXPERT    FLOOR 1  EARLY 100%  2.0b   2% 1.5c   LATE  100%  3.0b   5% 2.0c   ELITE 100%  3.4b   5% 2.0c   BOSS  100%  5.1b  11% 2.0c   </t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t xml:space="preserve">  EXPERT    FLOOR 2  EARLY 100%  3.2b   8% 2.0c   LATE  100%  3.3b  11% 2.0c   ELITE 100%  4.1b  14% 1.9c   BOSS  100%  6.2b  19% 2.0c   </t>
+          <t xml:space="preserve">  EXPERT    FLOOR 2  EARLY 100%  3.3b   8% 2.0c   LATE  100%  3.5b  11% 2.0c   ELITE 100%  4.1b  14% 2.0c   BOSS  100%  6.3b  19% 2.0c   </t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t xml:space="preserve">  EXPERT    FLOOR 3  EARLY 100%  3.9b  12% 2.0c   LATE  100%  4.8b  14% 2.0c   ELITE 100%  5.2b  22% 2.0c   BOSS   99%  7.6b  29% 2.0c   </t>
+          <t xml:space="preserve">  EXPERT    FLOOR 3  EARLY 100%  4.1b  13% 2.0c   LATE  100%  4.8b  15% 2.0c   ELITE 100%  5.2b  19% 2.0c   BOSS   99%  7.7b  31% 2.0c   </t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t xml:space="preserve">  STRONG    FLOOR 1  EARLY 100%  2.1b   6% 1.3c   LATE  100%  3.2b  14% 1.9c   ELITE 100%  3.7b  12% 1.8c   BOSS   98%  5.8b  26% 1.9c   </t>
+          <t xml:space="preserve">  STRONG    FLOOR 1  EARLY 100%  2.2b   6% 1.4c   LATE  100%  3.1b  11% 2.0c   ELITE 100%  3.7b  12% 1.9c   BOSS  100%  5.6b  24% 2.0c   </t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t xml:space="preserve">  STRONG    FLOOR 2  EARLY 100%  3.8b  20% 1.9c   LATE  100%  3.9b  25% 2.0c   ELITE  97%  4.9b  35% 1.9c   BOSS   87%  7.4b  49% 2.0c   </t>
+          <t xml:space="preserve">  STRONG    FLOOR 2  EARLY 100%  3.6b  17% 2.0c   LATE  100%  4.1b  25% 2.0c   ELITE 100%  4.7b  28% 2.0c   BOSS   87%  7.4b  50% 2.0c   </t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t xml:space="preserve">  STRONG    FLOOR 3  EARLY 100%  4.6b  26% 2.0c   LATE   99%  5.6b  38% 2.0c   ELITE  84%  6.3b  59% 2.0c   BOSS   56%  8.5b  76% 2.0c   </t>
+          <t xml:space="preserve">  STRONG    FLOOR 3  EARLY 100%  4.7b  29% 2.0c   LATE  100%  5.7b  39% 2.0c   ELITE  89%  6.5b  55% 2.0c   BOSS   56%  8.4b  75% 2.0c   </t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t xml:space="preserve">  AVERAGE   FLOOR 1  EARLY 100%  2.3b  12% 1.2c   LATE  100%  3.7b  28% 1.7c   ELITE 100%  4.2b  30% 1.7c   BOSS   79%  6.8b  55% 1.8c   </t>
+          <t xml:space="preserve">  AVERAGE   FLOOR 1  EARLY 100%  2.3b  10% 1.3c   LATE  100%  3.6b  23% 1.9c   ELITE 100%  4.2b  26% 1.9c   BOSS   84%  6.8b  53% 2.0c   </t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t xml:space="preserve">  AVERAGE   FLOOR 2  EARLY  96%  4.7b  42% 1.8c   LATE   70%  5.3b  70% 1.9c   ELITE  50%  5.6b  82% 1.7c   BOSS   19%  6.6b  93% 1.8c   </t>
+          <t xml:space="preserve">  AVERAGE   FLOOR 2  EARLY  99%  4.5b  37% 1.9c   LATE   77%  5.2b  65% 1.9c   ELITE  62%  5.8b  74% 1.9c   BOSS   21%  6.7b  91% 1.8c   </t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t xml:space="preserve">  AVERAGE   FLOOR 3  EARLY  52%  5.8b  80% 1.8c   LATE   16%  4.8b  95% 1.9c   ELITE   4%  4.2b  98% 1.7c   BOSS    1%  4.4b  99% 1.8c   </t>
+          <t xml:space="preserve">  AVERAGE   FLOOR 3  EARLY  56%  5.4b  76% 1.8c   LATE   16%  4.1b  95% 1.6c   ELITE   7%  4.4b  98% 1.6c   BOSS    1%  4.4b  99% 1.6c   </t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t xml:space="preserve">  NEWCOMER  FLOOR 1  EARLY 100%  2.5b  20% 1.1c   LATE   98%  4.2b  46% 1.6c   ELITE  98%  4.4b  44% 1.7c   BOSS   48%  6.8b  78% 1.7c   </t>
+          <t xml:space="preserve">  NEWCOMER  FLOOR 1  EARLY 100%  2.4b  15% 1.2c   LATE  100%  4.0b  34% 1.8c   ELITE  98%  4.5b  41% 1.9c   BOSS   47%  6.9b  78% 1.8c   </t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t xml:space="preserve">  NEWCOMER  FLOOR 2  EARLY  67%  5.3b  73% 1.7c   LATE    6%  3.7b  98% 1.4c   ELITE   6%  4.2b  98% 1.5c   BOSS    0%  4.1b  99% 1.4c   </t>
+          <t xml:space="preserve">  NEWCOMER  FLOOR 2  EARLY  86%  5.1b  62% 1.9c   LATE   18%  4.4b  94% 1.5c   ELITE   8%  4.6b  97% 1.7c   BOSS    0%  4.5b  99% 1.6c   </t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t xml:space="preserve">  NEWCOMER  FLOOR 3  EARLY   3%  3.4b  99% 1.5c   LATE    0%  2.4b 100% 1.4c   ELITE   0%  2.5b 100% 1.3c   BOSS    0%  2.5b 100% 1.3c   </t>
+          <t xml:space="preserve">  NEWCOMER  FLOOR 3  EARLY   2%  3.3b  98% 1.4c   LATE    0%  2.1b 100% 1.0c   ELITE   0%  2.4b 100% 1.2c   BOSS    0%  2.3b 100% 1.1c   </t>
         </is>
       </c>
     </row>
@@ -1621,49 +1621,49 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t xml:space="preserve">  HUSH                   74%  5.3b</t>
+          <t xml:space="preserve">  HUSH                   77%  5.2b</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t xml:space="preserve">  DEAD AIR               65%  5.2b</t>
+          <t xml:space="preserve">  DEAD AIR               74%  5.1b</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t xml:space="preserve">  THE LULL               75%  5.5b</t>
+          <t xml:space="preserve">  THE LULL               79%  5.5b</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t xml:space="preserve">  STATIC                 74%  5.2b</t>
+          <t xml:space="preserve">  STATIC                 79%  5.1b</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t xml:space="preserve">  THE MUTE CHOIR         68%  6.0b</t>
+          <t xml:space="preserve">  THE MUTE CHOIR         72%  6.1b</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t xml:space="preserve">  WHITE NOISE            33%  5.3b</t>
+          <t xml:space="preserve">  WHITE NOISE            47%  5.7b</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t xml:space="preserve">  REQUIEM                 0%  3.9b</t>
+          <t xml:space="preserve">  REQUIEM                 0%  3.8b</t>
         </is>
       </c>
     </row>
@@ -1677,153 +1677,188 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t xml:space="preserve">  THE DEVIL'S STRING      0%  3.3b</t>
-        </is>
-      </c>
-    </row>
-    <row r="32"/>
+          <t xml:space="preserve">  THE DEVIL'S STRING      0%  3.6b</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ROOM TONE              81%  5.5b</t>
+        </is>
+      </c>
+    </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>RUNS (3 floors, life carried over, no motifs) : WIN PERCENT  /  LOST ON FLOOR 1, 2, 3</t>
+          <t xml:space="preserve">  THE CUE                87%  5.3b</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t xml:space="preserve">  NORMAL</t>
+          <t xml:space="preserve">  THE DAMPER             68%  5.5b</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t xml:space="preserve">    FLAWLESS 100%    0% / 0% / 0%</t>
+          <t xml:space="preserve">  STUTTER                85%  5.2b</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t xml:space="preserve">    EXPERT   100%    0% / 0% / 0%</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    STRONG    56%    0% / 12% / 30%</t>
-        </is>
-      </c>
-    </row>
+          <t xml:space="preserve">  THE ROUND              68%  6.2b</t>
+        </is>
+      </c>
+    </row>
+    <row r="37"/>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t xml:space="preserve">    AVERAGE    0%    40% / 59% / 0%</t>
+          <t>RUNS (3 floors, life carried over, no motifs) : WIN PERCENT  /  LOST ON FLOOR 1, 2, 3</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t xml:space="preserve">    NEWCOMER   0%    92% / 7% / 0%</t>
+          <t xml:space="preserve">  NORMAL</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t xml:space="preserve">  MAESTRO</t>
+          <t xml:space="preserve">    FLAWLESS 100%    0% / 0% / 0%</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t xml:space="preserve">    FLAWLESS 100%    0% / 0% / 0%</t>
+          <t xml:space="preserve">    EXPERT   100%    0% / 0% / 0%</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t xml:space="preserve">    EXPERT    11%    9% / 45% / 34%</t>
+          <t xml:space="preserve">    STRONG    50%    0% / 10% / 38%</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t xml:space="preserve">    STRONG     0%    60% / 39% / 0%</t>
+          <t xml:space="preserve">    AVERAGE    0%    30% / 68% / 0%</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t xml:space="preserve">    AVERAGE    0%    100% / 0% / 0%</t>
+          <t xml:space="preserve">    NEWCOMER   0%    80% / 19% / 0%</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t xml:space="preserve">    NEWCOMER   0%    100% / 0% / 0%</t>
-        </is>
-      </c>
-    </row>
-    <row r="46"/>
+          <t xml:space="preserve">  MAESTRO</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    FLAWLESS 100%    0% / 0% / 0%</t>
+        </is>
+      </c>
+    </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>CONDUCTORS (runs as above, NORMAL) : WIN PERCENT  STRONG / AVERAGE</t>
+          <t xml:space="preserve">    EXPERT    79%    0% / 3% / 17%</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t xml:space="preserve">  THE UNHEARING       58% / 0%</t>
+          <t xml:space="preserve">    STRONG     0%    15% / 72% / 12%</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t xml:space="preserve">  THE SHADOWLESS      55% / 0%</t>
+          <t xml:space="preserve">    AVERAGE    0%    94% / 5% / 0%</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t xml:space="preserve">  THE METRONOME       44% / 0%</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  THE HEARTLESS       64% / 0%</t>
-        </is>
-      </c>
-    </row>
+          <t xml:space="preserve">    NEWCOMER   0%    100% / 0% / 0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="51"/>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t xml:space="preserve">  THE KING'S BATON    66% / 0%</t>
+          <t>CONDUCTORS (runs as above, NORMAL) : WIN PERCENT  STRONG / AVERAGE</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t xml:space="preserve">  THE UNSIGNED        45% / 0%</t>
-        </is>
-      </c>
-    </row>
-    <row r="54"/>
+          <t xml:space="preserve">  THE UNHEARING       58% / 0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  THE SHADOWLESS      51% / 0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  THE METRONOME       51% / 0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  THE HEARTLESS       65% / 0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  THE KING'S BATON    63% / 0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  THE UNSIGNED        50% / 0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="59"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -8612,7 +8647,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D131"/>
+  <dimension ref="A1:D140"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" style="33" min="1" max="1"/>
@@ -9344,134 +9379,144 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>PRACTICE</t>
+          <t>ONE BAR enemies</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>TurnPracticeHp</t>
+          <t>TurnRoomToneKeep</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>160</t>
+          <t>0.7</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>ROOM TONE : the share of the band's damage the OTHER enemies take while it stands</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>PRACTICE</t>
+          <t>ONE BAR enemies</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>TurnPracticeSpeed</t>
+          <t>TurnFeltHandCall</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>THE DAMPER : a CALL costs this much more while it stands (2 left the sim's STRONG player at 23 percent against it)</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>PRACTICE</t>
+          <t>ONE BAR enemies</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>TurnPracticePower</t>
+          <t>TurnTwiceFirst</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>each note hits this x TurnNoteDamage (4 life)</t>
+          <t>STUTTER : cuts in after this many of the band's moves</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Enemy Attack</t>
+          <t>ONE BAR enemies</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>TurnNotesMin</t>
+          <t>TurnTwiceSecond</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>{ 1, 2, 3 }</t>
+          <t>3</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>ELITE and BOSS</t>
+          <t>and again after this many</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Enemy Attack</t>
+          <t>PRACTICE</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>TurnNotesMax</t>
+          <t>TurnPracticeHp</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>{ 2, 3, 4 }</t>
+          <t>160</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Enemy Attack</t>
+          <t>PRACTICE</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>TurnSmallNotesMin</t>
+          <t>TurnPracticeSpeed</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>{ 1, 1, 2 }</t>
-        </is>
-      </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>ordinary enemies</t>
+          <t>4</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Enemy Attack</t>
+          <t>PRACTICE</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>TurnSmallNotesMax</t>
+          <t>TurnPracticePower</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>{ 2, 2, 2 }</t>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>each note hits this x TurnNoteDamage (4 life)</t>
         </is>
       </c>
     </row>
@@ -9483,268 +9528,263 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>TurnNoteDamage</t>
+          <t>TurnNotesMin</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>2.2</t>
+          <t>{ 1, 2, 3 }</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>step 12 : was 1.5, the user found NORMAL far too easy (turnsim STRONG 81 -&gt; 57 percent)</t>
+          <t>ELITE and BOSS</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>PARRY</t>
+          <t>Enemy Attack</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>TurnParryGoodKeep</t>
+          <t>TurnNotesMax</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>0.5</t>
+          <t>{ 2, 3, 4 }</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>BREATH</t>
+          <t>Enemy Attack</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>TurnBreathMax</t>
+          <t>TurnSmallNotesMin</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>{ 1, 1, 2 }</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>ordinary enemies</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>BREATH</t>
+          <t>Enemy Attack</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>TurnBreathStart</t>
+          <t>TurnSmallNotesMax</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>{ 2, 2, 2 }</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>BREATH</t>
+          <t>Enemy Attack</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>TurnBreathPerAttack</t>
+          <t>TurnNoteDamage</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2.2</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>step 12 : was 1.5, the user found NORMAL far too easy (turnsim STRONG 81 -&gt; 57 percent)</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>BREATH</t>
+          <t>PARRY</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>TurnBreathPerParry</t>
+          <t>TurnParryGoodKeep</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="D48" t="inlineStr">
-        <is>
-          <t>for each note parried PERFECT</t>
+          <t>0.5</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>KNOCKED OUT</t>
+          <t>BREATH</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>TurnReviveHp</t>
+          <t>TurnBreathMax</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>10</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>OFF-BEAT</t>
+          <t>BREATH</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>TurnOffBeatMax</t>
+          <t>TurnBreathStart</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>3</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>OFF-BEAT</t>
+          <t>BREATH</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>TurnParryOffBeat</t>
+          <t>TurnBreathPerAttack</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="D51" t="inlineStr">
-        <is>
-          <t>each note parried PERFECT</t>
+          <t>1</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>OFF-BEAT</t>
+          <t>BREATH</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>TurnOffBeatScale</t>
+          <t>TurnBreathPerParry</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>1.5</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>damage against an enemy off the beat</t>
+          <t>for each note parried PERFECT</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Statuses</t>
+          <t>KNOCKED OUT</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>TurnDissonanceMost</t>
+          <t>TurnReviveHp</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>9</t>
-        </is>
-      </c>
-      <c r="D53" t="inlineStr">
-        <is>
-          <t>DISSONANCE stacks no higher</t>
+          <t>1</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Statuses</t>
+          <t>OFF-BEAT</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>TurnCrescendoStep</t>
+          <t>TurnOffBeatMax</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>0.15</t>
-        </is>
-      </c>
-      <c r="D54" t="inlineStr">
-        <is>
-          <t>CRESCENDO : each stack hits this much harder</t>
+          <t>100</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Statuses</t>
+          <t>OFF-BEAT</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>TurnCrescendoMost</t>
+          <t>TurnParryOffBeat</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>each note parried PERFECT</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Statuses</t>
+          <t>OFF-BEAT</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>TurnMuteTurns</t>
+          <t>TurnOffBeatScale</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>1.5</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>MUTE : turns without skills</t>
+          <t>damage against an enemy off the beat</t>
         </is>
       </c>
     </row>
@@ -9756,158 +9796,173 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>TurnGuardKeep</t>
+          <t>TurnDissonanceMost</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>0.5</t>
+          <t>9</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>GUARD : the share of a hit that gets through</t>
+          <t>DISSONANCE stacks no higher</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>COUNTER and CADENZA</t>
+          <t>Statuses</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>TurnCounterScale</t>
+          <t>TurnCrescendoStep</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0.15</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>x the target's attack damage</t>
+          <t>CRESCENDO : each stack hits this much harder</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>COUNTER and CADENZA</t>
+          <t>Statuses</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>TurnCadenzaCounter</t>
+          <t>TurnCrescendoMost</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>COUNTER and CADENZA</t>
+          <t>Statuses</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>TurnCadenzaEvery</t>
+          <t>TurnMuteTurns</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>MUTE : turns without skills</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>COUNTER and CADENZA</t>
+          <t>Statuses</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>TurnCadenzaPower</t>
+          <t>TurnGuardKeep</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>1.5</t>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>GUARD : the share of a hit that gets through</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Skill Notes</t>
+          <t>COUNTER and CADENZA</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>TurnHoldBase</t>
+          <t>TurnCounterScale</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>0.6</t>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>x the target's attack damage</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Skill Notes</t>
+          <t>COUNTER and CADENZA</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>TurnHoldGain</t>
+          <t>TurnCadenzaCounter</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>0.8</t>
+          <t>2</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Skill Notes</t>
+          <t>COUNTER and CADENZA</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>TurnRollPerfect</t>
+          <t>TurnCadenzaEvery</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Skill Notes</t>
+          <t>COUNTER and CADENZA</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>TurnRollGood</t>
+          <t>TurnCadenzaPower</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1.5</t>
         </is>
       </c>
     </row>
@@ -9919,12 +9974,12 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>MaestroTurnRollPerfect</t>
+          <t>TurnHoldBase</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>0.6</t>
         </is>
       </c>
     </row>
@@ -9936,95 +9991,80 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>MaestroTurnRollGood</t>
+          <t>TurnHoldGain</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>0.8</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Conductors</t>
+          <t>Skill Notes</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>TurnSignatureNeed</t>
+          <t>TurnRollPerfect</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Conductors</t>
+          <t>Skill Notes</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>TurnBeethovenMost</t>
+          <t>TurnRollGood</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>0.5</t>
-        </is>
-      </c>
-      <c r="D69" t="inlineStr">
-        <is>
-          <t>THE UNHEARING's PASSIVE : up to this much harder as the band's life runs out</t>
+          <t>3</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Conductors</t>
+          <t>Skill Notes</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>TurnBoltDamage</t>
+          <t>MaestroTurnRollPerfect</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>14</t>
-        </is>
-      </c>
-      <c r="D70" t="inlineStr">
-        <is>
-          <t>LIGHTNING : damage to every enemy at full strength (x1)</t>
+          <t>6</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Conductors</t>
+          <t>Skill Notes</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>TurnMozartRun</t>
+          <t>MaestroTurnRollGood</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="D71" t="inlineStr">
-        <is>
-          <t>THE SHADOWLESS's PASSIVE : this many PERFECTs in a row give 1 breath</t>
+          <t>4</t>
         </is>
       </c>
     </row>
@@ -10036,105 +10076,100 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>TurnFeatherPerStroke</t>
+          <t>TurnSignatureNeed</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="D72" t="inlineStr">
-        <is>
-          <t>FEATHER : free ATTACKs per stroke that lands (step 12, was 1 extra turn : 25 percent of STRONG runs won)</t>
+          <t>6</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>The other four of the lore</t>
+          <t>Conductors</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>TurnPaganiniLife</t>
+          <t>TurnBeethovenMost</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>0.5</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>THE HEARTLESS's PASSIVE : life paid for each BREATH a skill is short of</t>
+          <t>THE UNHEARING's PASSIVE : up to this much harder as the band's life runs out</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>The other four of the lore</t>
+          <t>Conductors</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>TurnCapricePrice</t>
+          <t>TurnBoltDamage</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>0.1</t>
+          <t>14</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>CAPRICE : when it ends, every musician pays this share of their life (never below 1)</t>
+          <t>LIGHTNING : damage to every enemy at full strength (x1)</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>The other four of the lore</t>
+          <t>Conductors</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>TurnCapricePerStroke</t>
+          <t>TurnMozartRun</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>CAPRICE : turns per stroke that lands (step 12, a bar has more turns now)</t>
+          <t>THE SHADOWLESS's PASSIVE : this many PERFECTs in a row give 1 breath</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>The other four of the lore</t>
+          <t>Conductors</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>TurnLullyWindow</t>
+          <t>TurnFeatherPerStroke</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>0.01</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>THE KING'S BATON's PASSIVE : seconds added to both parry windows (0.05 won 99 percent of STRONG runs, the others 83 to 90;</t>
+          <t>FEATHER : free ATTACKs per stroke that lands (step 12, was 1 extra turn : 25 percent of STRONG runs won)</t>
         </is>
       </c>
     </row>
@@ -10146,17 +10181,17 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>TurnSunHeal</t>
+          <t>TurnFugueScale</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>1.8</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>THE SUN : life back for every musician at full strength</t>
+          <t>FUGUE : the echo plays at the SIGNATURE's strength x this (step 13 : was 1, THE METRONOME was the weakest at 44 percent)</t>
         </is>
       </c>
     </row>
@@ -10168,17 +10203,17 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>TurnFannyScale</t>
+          <t>TurnPaganiniLife</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>0.25</t>
+          <t>3</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>THE UNSIGNED's PASSIVE : FANNY's voice hits this much harder</t>
+          <t>THE HEARTLESS's PASSIVE : life paid for each BREATH a skill is short of</t>
         </is>
       </c>
     </row>
@@ -10190,17 +10225,17 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>TurnFelixHeal</t>
+          <t>TurnCapricePrice</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>1.5</t>
+          <t>0.2</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>FELIX's voice heals this much more</t>
+          <t>CAPRICE : when it ends, every musician pays this share of their life (never below 1, step 13 : was 0.1)</t>
         </is>
       </c>
     </row>
@@ -10212,17 +10247,17 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>TurnFelixCrescendo</t>
+          <t>TurnCapricePerStroke</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>and gives this much more CRESCENDO</t>
+          <t>CAPRICE : turns per stroke that lands (step 12, a bar has more turns now)</t>
         </is>
       </c>
     </row>
@@ -10234,17 +10269,17 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>TurnDuetDamage</t>
+          <t>TurnLullyWindow</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>0.01</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>TWO VOICES : damage to every enemy at full strength</t>
+          <t>THE KING'S BATON's PASSIVE : seconds added to both parry windows (0.05 won 99 percent of STRONG runs, the others 83 to 90;</t>
         </is>
       </c>
     </row>
@@ -10256,51 +10291,51 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>TurnDuetHeal</t>
+          <t>TurnSunHeal</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>8</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>and life back for every musician</t>
+          <t>THE SUN : life back for every musician at full strength (step 13 : was 12, THE KING'S BATON was the strongest at 71 percent)</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Musician Traits in the turn battle</t>
+          <t>The other four of the lore</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>TurnCountsWindow</t>
+          <t>TurnFannyScale</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>0.05</t>
+          <t>0.25</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>COUNTS ALOUD (ANNA) : seconds added to her PERFECT window</t>
+          <t>THE UNSIGNED's PASSIVE : FANNY's voice hits this much harder</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>Musician Traits in the turn battle</t>
+          <t>The other four of the lore</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>TurnQuietScale</t>
+          <t>TurnFelixHeal</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
@@ -10310,73 +10345,73 @@
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>THE QUIET PART (KLARA) : against an enemy showing a p note</t>
+          <t>FELIX's voice heals this much more</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>Musician Traits in the turn battle</t>
+          <t>The other four of the lore</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>TurnMomentumMost</t>
+          <t>TurnFelixCrescendo</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>MOMENTUM (OTTO) : power gained by hits in a row, at most</t>
+          <t>and gives this much more CRESCENDO</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>Musician Traits in the turn battle</t>
+          <t>The other four of the lore</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>TurnByEarScale</t>
+          <t>TurnDuetDamage</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>1.5</t>
+          <t>12</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>BY EAR (MALI) : against an enemy that is OFF-BEAT</t>
+          <t>TWO VOICES : damage to every enemy at full strength (step 13 : was 9 and 6, THE UNSIGNED 46 percent)</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>Musician Traits in the turn battle</t>
+          <t>The other four of the lore</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>TurnHeldNoteShare</t>
+          <t>TurnDuetHeal</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>0.4</t>
+          <t>8</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>HELD NOTE (CHAI) : his ATTACK hits again for this share</t>
+          <t>and life back for every musician</t>
         </is>
       </c>
     </row>
@@ -10388,17 +10423,17 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>TurnStepBetterScale</t>
+          <t>TurnCountsWindow</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>1.3</t>
+          <t>0.05</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>ONE STEP BETTER (NUAN) : against an enemy showing an f note</t>
+          <t>COUNTS ALOUD (ANNA) : seconds added to her PERFECT window</t>
         </is>
       </c>
     </row>
@@ -10410,17 +10445,17 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>TurnFourBarsEvery</t>
+          <t>TurnQuietScale</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1.5</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>FOUR BARS STRAIGHT (LUKA) : every this many ATTACKs</t>
+          <t>THE QUIET PART (KLARA) : against an enemy showing a p note</t>
         </is>
       </c>
     </row>
@@ -10432,17 +10467,17 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>TurnFourBarsScale</t>
+          <t>TurnMomentumMost</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>hits this much harder</t>
+          <t>MOMENTUM (OTTO) : power gained by hits in a row, at most</t>
         </is>
       </c>
     </row>
@@ -10454,17 +10489,17 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>TurnLateBonus</t>
+          <t>TurnByEarScale</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>0.12</t>
+          <t>1.5</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>FASHIONABLY LATE (IRIS) : seconds after the GOOD window a late stroke still counts</t>
+          <t>BY EAR (MALI) : against an enemy that is OFF-BEAT</t>
         </is>
       </c>
     </row>
@@ -10476,117 +10511,117 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>TurnThunderSoften</t>
+          <t>TurnHeldNoteShare</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0.4</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>THE WHOLE FLOOR (BORIS) : taken off each note of the enemy's next attack</t>
+          <t>HELD NOTE (CHAI) : his ATTACK hits again for this share</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>ARCHIVE</t>
+          <t>Musician Traits in the turn battle</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>EchoesPerWin</t>
+          <t>TurnStepBetterScale</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1.3</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>each fight won</t>
+          <t>ONE STEP BETTER (NUAN) : against an enemy showing an f note</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>ARCHIVE</t>
+          <t>Musician Traits in the turn battle</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>EchoesPerFloor</t>
+          <t>TurnFourBarsEvery</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>4</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>each floor cleared</t>
+          <t>FOUR BARS STRAIGHT (LUKA) : every this many ATTACKs</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>ARCHIVE</t>
+          <t>Musician Traits in the turn battle</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>EchoesRunWon</t>
+          <t>TurnFourBarsScale</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>the whole run won</t>
+          <t>hits this much harder</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>ARCHIVE</t>
+          <t>Musician Traits in the turn battle</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>EchoesMaestro</t>
+          <t>TurnLateBonus</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>1.5</t>
+          <t>0.12</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>MAESTRO pays more</t>
+          <t>FASHIONABLY LATE (IRIS) : seconds after the GOOD window a late stroke still counts</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>ARCHIVE</t>
+          <t>Musician Traits in the turn battle</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>ArchiveLifePerLevel</t>
+          <t>TurnThunderSoften</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
@@ -10596,7 +10631,7 @@
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>STRONGER BAND</t>
+          <t>THE WHOLE FLOOR (BORIS) : taken off each note of the enemy's next attack</t>
         </is>
       </c>
     </row>
@@ -10608,17 +10643,17 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>ArchiveBreathPerLevel</t>
+          <t>EchoesPerWin</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>DEEP BREATH</t>
+          <t>each fight won</t>
         </is>
       </c>
     </row>
@@ -10630,17 +10665,17 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>ArchiveSignaturePerLevel</t>
+          <t>EchoesPerFloor</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>10</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>WARM UP</t>
+          <t>each floor cleared</t>
         </is>
       </c>
     </row>
@@ -10652,17 +10687,17 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>ArchiveShardsPerLevel</t>
+          <t>EchoesRunWon</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>25</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>SAVINGS</t>
+          <t>the whole run won</t>
         </is>
       </c>
     </row>
@@ -10674,127 +10709,127 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>ArchiveStagePerLevel</t>
+          <t>EchoesMaestro</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>1.5</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>FULL STAGE : musicians more on the field at the start (step 12)</t>
+          <t>MAESTRO pays more</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>Turn Motifs</t>
+          <t>ARCHIVE</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>TurnReedCaseHeal</t>
+          <t>ArchiveLifePerLevel</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>1.5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>REED CASE : wind players' healing</t>
+          <t>STRONGER BAND</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>Turn Motifs</t>
+          <t>ARCHIVE</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>TurnSpareSticksOffBeat</t>
+          <t>ArchiveBreathPerLevel</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>1.5</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>SPARE STICKS : percussion skills' OFF-BEAT</t>
+          <t>DEEP BREATH</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>Turn Motifs</t>
+          <t>ARCHIVE</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>TurnPianissimoBreath</t>
+          <t>ArchiveSignaturePerLevel</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>PIANISSIMO : more breath for a p note parried PERFECT</t>
+          <t>WARM UP</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>Turn Motifs</t>
+          <t>ARCHIVE</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>TurnBreathMarkStart</t>
+          <t>ArchiveShardsPerLevel</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>20</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>BREATH MARK : more breath at the start of a fight</t>
+          <t>SAVINGS</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>Turn Motifs</t>
+          <t>ARCHIVE</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>TurnTuttiScale</t>
+          <t>ArchiveStagePerLevel</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>1.25</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>TUTTI : skills that reach everyone</t>
+          <t>FULL STAGE : musicians more on the field at the start (step 12)</t>
         </is>
       </c>
     </row>
@@ -10806,17 +10841,17 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>TurnRubatoMiss</t>
+          <t>TurnReedCaseHeal</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>0.6</t>
+          <t>1.5</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>RUBATO : a skill note you MISS still plays at this (step 12)</t>
+          <t>REED CASE : wind players' healing</t>
         </is>
       </c>
     </row>
@@ -10828,17 +10863,17 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>TurnCrescendoStart</t>
+          <t>TurnSpareSticksOffBeat</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>1.5</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>CRESCENDO : stacks on every musician at the start</t>
+          <t>SPARE STICKS : percussion skills' OFF-BEAT</t>
         </is>
       </c>
     </row>
@@ -10850,17 +10885,17 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>TurnSforzandoScale</t>
+          <t>TurnPianissimoBreath</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>1.3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>SFORZANDO : a PERFECT f note</t>
+          <t>PIANISSIMO : more breath for a p note parried PERFECT</t>
         </is>
       </c>
     </row>
@@ -10872,7 +10907,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>TurnOvertureScale</t>
+          <t>TurnBreathMarkStart</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
@@ -10882,7 +10917,7 @@
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>OVERTURE : the band's first hit of a fight</t>
+          <t>BREATH MARK : more breath at the start of a fight</t>
         </is>
       </c>
     </row>
@@ -10894,17 +10929,17 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>TurnCounterpointScale</t>
+          <t>TurnTuttiScale</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1.25</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>COUNTERPOINT : the COUNTER</t>
+          <t>TUTTI : skills that reach everyone</t>
         </is>
       </c>
     </row>
@@ -10916,17 +10951,17 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>TurnAccelerandoShakes</t>
+          <t>TurnRubatoMiss</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0.6</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>ACCELERANDO : each shake of a roll counts this many</t>
+          <t>RUBATO : a skill note you MISS still plays at this (step 12)</t>
         </is>
       </c>
     </row>
@@ -10938,17 +10973,17 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>TurnGraceTimes</t>
+          <t>TurnCrescendoStart</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>GRACE NOTE : a spark that lands does its skill this many times</t>
+          <t>CRESCENDO : stacks on every musician at the start</t>
         </is>
       </c>
     </row>
@@ -10960,17 +10995,17 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>TurnMarcatoOffBeat</t>
+          <t>TurnSforzandoScale</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1.3</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>MARCATO : a PERFECT attack's OFF-BEAT, times this</t>
+          <t>SFORZANDO : a PERFECT f note</t>
         </is>
       </c>
     </row>
@@ -10982,17 +11017,17 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>TurnConBrioNeed</t>
+          <t>TurnOvertureScale</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>CON BRIO : PERFECTs the SIGNATURE needs instead</t>
+          <t>OVERTURE : the band's first hit of a fight</t>
         </is>
       </c>
     </row>
@@ -11004,17 +11039,17 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>TurnCodaBelow</t>
+          <t>TurnCounterpointScale</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>0.25</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>CODA : an enemy under this share of its life</t>
+          <t>COUNTERPOINT : the COUNTER</t>
         </is>
       </c>
     </row>
@@ -11026,215 +11061,215 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>TurnCodaScale</t>
+          <t>TurnAccelerandoShakes</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>1.5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>takes this much more</t>
+          <t>ACCELERANDO : each shake of a roll counts this many</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>Turn Feel</t>
+          <t>Turn Motifs</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>TurnRingTime</t>
+          <t>TurnGraceTimes</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>1.1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>from a note showing to the moment to swipe</t>
+          <t>GRACE NOTE : a spark that lands does its skill this many times</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>Turn Feel</t>
+          <t>Turn Motifs</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>MaestroTurnRingTime</t>
+          <t>TurnMarcatoOffBeat</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>0.8</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>MAESTRO</t>
+          <t>MARCATO : a PERFECT attack's OFF-BEAT, times this</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>Turn Feel</t>
+          <t>Turn Motifs</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>TurnNoteGap</t>
+          <t>TurnConBrioNeed</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>0.55</t>
+          <t>4</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>between the notes of one enemy attack</t>
+          <t>CON BRIO : PERFECTs the SIGNATURE needs instead</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>Turn Feel</t>
+          <t>Turn Motifs</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>TurnPause</t>
+          <t>TurnCodaBelow</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>0.8</t>
+          <t>0.25</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>after a turn, before the next one starts</t>
+          <t>CODA : an enemy under this share of its life</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>Turn Feel</t>
+          <t>Turn Motifs</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>TurnHitStop</t>
+          <t>TurnCodaScale</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>0.075</t>
+          <t>1.5</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>the band and TACET freeze for a moment on a PERFECT</t>
+          <t>takes this much more</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>Turn Feel</t>
+          <t>ONE BAR motifs</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>TurnStrikeTime</t>
+          <t>TurnDownbeatScale</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>0.42</t>
+          <t>1.5</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>ONE BAR : how long an ATTACK's lunge takes, there and back</t>
+          <t>DOWNBEAT : the first move of a bar</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>Turn Feel</t>
+          <t>ONE BAR motifs</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>TurnStrikeImpact</t>
+          <t>TurnEntranceScale</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>0.16</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>when in it the hit lands</t>
+          <t>ENTRANCE : a called musician's moves in their first bar</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>Turn Feel</t>
+          <t>ONE BAR motifs</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>TurnStrikeStop</t>
+          <t>TurnGreenRoomHeal</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>0.07</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>the freeze when it lands</t>
+          <t>GREEN ROOM : life back for each musician on the BENCH at the end of a bar</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>Turn Feel</t>
+          <t>ONE BAR motifs</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>TurnKillStop</t>
+          <t>TurnUnisonScale</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>0.18</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>the freeze when an enemy falls silent</t>
+          <t>UNISON : the last ATTACK of a bar that all goes at one enemy</t>
         </is>
       </c>
     </row>
@@ -11246,17 +11281,17 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>TurnEndTime</t>
+          <t>TurnRingTime</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>2.2</t>
+          <t>1.1</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>the win or lose banner stays this long</t>
+          <t>from a note showing to the moment to swipe</t>
         </is>
       </c>
     </row>
@@ -11268,17 +11303,17 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>TurnSparkGap</t>
+          <t>MaestroTurnRingTime</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>0.3</t>
+          <t>0.8</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>a spark comes this soon after the note before it</t>
+          <t>MAESTRO</t>
         </is>
       </c>
     </row>
@@ -11290,17 +11325,17 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>TurnHoldTime</t>
+          <t>TurnNoteGap</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>0.8</t>
+          <t>0.55</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>how long a HOLD note wants holding</t>
+          <t>between the notes of one enemy attack</t>
         </is>
       </c>
     </row>
@@ -11312,17 +11347,17 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>TurnHoldStill</t>
+          <t>TurnPause</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>0.8</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>pixels per second the baton may drift and still count as still</t>
+          <t>after a turn, before the next one starts</t>
         </is>
       </c>
     </row>
@@ -11334,15 +11369,213 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
+          <t>TurnHitStop</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>0.075</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>the band and TACET freeze for a moment on a PERFECT</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>Turn Feel</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>TurnStrikeTime</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>0.42</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>ONE BAR : how long an ATTACK's lunge takes, there and back</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>Turn Feel</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>TurnStrikeImpact</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>0.16</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>when in it the hit lands</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>Turn Feel</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>TurnStrikeStop</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>0.07</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>the freeze when it lands</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>Turn Feel</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>TurnKillStop</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>0.18</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>the freeze when an enemy falls silent</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>Turn Feel</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>TurnEndTime</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>2.2</t>
+        </is>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>the win or lose banner stays this long</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>Turn Feel</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>TurnSparkGap</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>0.3</t>
+        </is>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>a spark comes this soon after the note before it</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>Turn Feel</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>TurnHoldTime</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>0.8</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>how long a HOLD note wants holding</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>Turn Feel</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>TurnHoldStill</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>260</t>
+        </is>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>pixels per second the baton may drift and still count as still</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>Turn Feel</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
           <t>TurnRollTime</t>
         </is>
       </c>
-      <c r="C131" t="inlineStr">
+      <c r="C140" t="inlineStr">
         <is>
           <t>1.2</t>
         </is>
       </c>
-      <c r="D131" t="inlineStr">
+      <c r="D140" t="inlineStr">
         <is>
           <t>how long a ROLL note lasts</t>
         </is>
@@ -11359,7 +11592,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I10"/>
+  <dimension ref="A1:I15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" style="33" min="1" max="1"/>
@@ -11804,6 +12037,219 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>ROOM TONE</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>45</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>4</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Dp, Up Dp</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>HOLDS THE ROOM (2)</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>While it stands, the other enemies take 30 percent less.</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>THE CUE</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>55</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>4</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Rmf Lmf, Uf</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>ON CUE (2)</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>It always strikes the musician who was CALLED in last.</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>THE DAMPER</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>42</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>4</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Dmf Dp, Lmf Rmf</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>FELT HAND (2)</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>While it stands, a CALL costs 1 more BREATH.</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>STUTTER</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>36</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>4</v>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Lp, Rp, Up</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>TWICE A BAR (2)</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>It cuts in twice a bar, after the 1st and the 3rd move, one note each time.</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>THE ROUND</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Elite</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>115</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>5</v>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Df Dmf Df, Lmf Rmf Lf Rf</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>FIRST IN LINE (1)</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>It always strikes the musician who plays first in the bar.</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Alpha7 step 14: three bosses (option B) and the wrong-way swipe fix
- each era picks one of two bosses: THE DEAF CROWN (DECREE, no COUNTER),
  THE STAFF (THE COURT, every third attack hits everyone),
  THE BLIND CANTOR (BY TOUCH, seats in turn, missed notes come back)
- swipes: a stroke that would be a MISS (wrong way or too early) waits until
  the note's window closes, so the hand going back to the middle with the
  button held is no longer taken as the next note; the pointer is moved to
  the middle when a swipe starts so the screen edge cannot cut it short
- turnsim shows STRONG next to AVERAGE per enemy and obeys the DECREE;
  turncheck 113/113, shots battlecrown battlestaff battlecantor

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WqLsaY7gVTeQY89VfVgASG
</commit_message>
<xml_diff>
--- a/docs/TACET_Balance.xlsx
+++ b/docs/TACET_Balance.xlsx
@@ -1470,7 +1470,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A59"/>
+  <dimension ref="A1:A62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="140" customWidth="1" style="33" min="1" max="1"/>
@@ -1508,105 +1508,105 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t xml:space="preserve">  FLAWLESS  FLOOR 1  EARLY 100%  2.0b   0% 1.8c   LATE  100%  2.9b   0% 2.0c   ELITE 100%  3.0b   0% 1.9c   BOSS  100%  4.9b   0% 2.0c   </t>
+          <t xml:space="preserve">  FLAWLESS  FLOOR 1  EARLY 100%  2.0b   0% 1.8c   LATE  100%  2.9b   0% 2.0c   ELITE 100%  3.0b   0% 1.9c   BOSS  100%  5.0b   0% 2.0c   </t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t xml:space="preserve">  FLAWLESS  FLOOR 2  EARLY 100%  3.0b   0% 2.0c   LATE  100%  3.2b   0% 2.0c   ELITE 100%  3.9b   0% 2.0c   BOSS  100%  5.7b   0% 2.0c   </t>
+          <t xml:space="preserve">  FLAWLESS  FLOOR 2  EARLY 100%  3.0b   0% 2.0c   LATE  100%  3.2b   0% 2.0c   ELITE 100%  3.9b   0% 2.0c   BOSS  100%  5.9b   0% 2.0c   </t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t xml:space="preserve">  FLAWLESS  FLOOR 3  EARLY 100%  3.9b   0% 2.0c   LATE  100%  4.2b   0% 2.0c   ELITE 100%  4.4b   0% 2.0c   BOSS  100%  6.9b   0% 2.0c   </t>
+          <t xml:space="preserve">  FLAWLESS  FLOOR 3  EARLY 100%  3.8b   0% 2.0c   LATE  100%  4.2b   0% 2.0c   ELITE 100%  4.4b   0% 2.0c   BOSS  100%  7.0b   1% 2.0c   </t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t xml:space="preserve">  EXPERT    FLOOR 1  EARLY 100%  2.0b   2% 1.5c   LATE  100%  3.0b   5% 2.0c   ELITE 100%  3.4b   5% 2.0c   BOSS  100%  5.1b  11% 2.0c   </t>
+          <t xml:space="preserve">  EXPERT    FLOOR 1  EARLY 100%  2.1b   2% 1.5c   LATE  100%  3.0b   5% 2.0c   ELITE 100%  3.4b   5% 2.0c   BOSS  100%  5.1b  12% 2.0c   </t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t xml:space="preserve">  EXPERT    FLOOR 2  EARLY 100%  3.3b   8% 2.0c   LATE  100%  3.5b  11% 2.0c   ELITE 100%  4.1b  14% 2.0c   BOSS  100%  6.3b  19% 2.0c   </t>
+          <t xml:space="preserve">  EXPERT    FLOOR 2  EARLY 100%  3.2b   8% 1.9c   LATE  100%  3.6b  11% 2.0c   ELITE 100%  4.2b  14% 2.0c   BOSS  100%  6.2b  20% 2.0c   </t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t xml:space="preserve">  EXPERT    FLOOR 3  EARLY 100%  4.1b  13% 2.0c   LATE  100%  4.8b  15% 2.0c   ELITE 100%  5.2b  19% 2.0c   BOSS   99%  7.7b  31% 2.0c   </t>
+          <t xml:space="preserve">  EXPERT    FLOOR 3  EARLY 100%  4.0b  12% 2.0c   LATE  100%  4.8b  15% 2.0c   ELITE 100%  5.1b  19% 2.0c   BOSS  100%  7.7b  29% 2.0c   </t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t xml:space="preserve">  STRONG    FLOOR 1  EARLY 100%  2.2b   6% 1.4c   LATE  100%  3.1b  11% 2.0c   ELITE 100%  3.7b  12% 1.9c   BOSS  100%  5.6b  24% 2.0c   </t>
+          <t xml:space="preserve">  STRONG    FLOOR 1  EARLY 100%  2.1b   5% 1.4c   LATE  100%  3.2b  11% 2.0c   ELITE 100%  3.7b  12% 1.9c   BOSS  100%  5.6b  25% 2.0c   </t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t xml:space="preserve">  STRONG    FLOOR 2  EARLY 100%  3.6b  17% 2.0c   LATE  100%  4.1b  25% 2.0c   ELITE 100%  4.7b  28% 2.0c   BOSS   87%  7.4b  50% 2.0c   </t>
+          <t xml:space="preserve">  STRONG    FLOOR 2  EARLY 100%  3.8b  18% 1.9c   LATE  100%  4.2b  23% 2.0c   ELITE 100%  4.8b  28% 2.0c   BOSS   91%  7.3b  51% 2.0c   </t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t xml:space="preserve">  STRONG    FLOOR 3  EARLY 100%  4.7b  29% 2.0c   LATE  100%  5.7b  39% 2.0c   ELITE  89%  6.5b  55% 2.0c   BOSS   56%  8.4b  75% 2.0c   </t>
+          <t xml:space="preserve">  STRONG    FLOOR 3  EARLY 100%  4.8b  28% 2.0c   LATE   98%  5.7b  40% 2.0c   ELITE  88%  6.5b  56% 2.0c   BOSS   53%  8.2b  78% 2.0c   </t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t xml:space="preserve">  AVERAGE   FLOOR 1  EARLY 100%  2.3b  10% 1.3c   LATE  100%  3.6b  23% 1.9c   ELITE 100%  4.2b  26% 1.9c   BOSS   84%  6.8b  53% 2.0c   </t>
+          <t xml:space="preserve">  AVERAGE   FLOOR 1  EARLY 100%  2.3b  10% 1.3c   LATE  100%  3.5b  22% 1.9c   ELITE 100%  4.1b  24% 1.9c   BOSS   87%  7.1b  62% 2.0c   </t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t xml:space="preserve">  AVERAGE   FLOOR 2  EARLY  99%  4.5b  37% 1.9c   LATE   77%  5.2b  65% 1.9c   ELITE  62%  5.8b  74% 1.9c   BOSS   21%  6.7b  91% 1.8c   </t>
+          <t xml:space="preserve">  AVERAGE   FLOOR 2  EARLY  98%  4.4b  39% 1.9c   LATE   78%  5.4b  67% 1.9c   ELITE  67%  5.9b  73% 1.9c   BOSS   13%  6.2b  95% 1.9c   </t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t xml:space="preserve">  AVERAGE   FLOOR 3  EARLY  56%  5.4b  76% 1.8c   LATE   16%  4.1b  95% 1.6c   ELITE   7%  4.4b  98% 1.6c   BOSS    1%  4.4b  99% 1.6c   </t>
+          <t xml:space="preserve">  AVERAGE   FLOOR 3  EARLY  52%  5.3b  80% 1.8c   LATE   17%  4.3b  93% 1.6c   ELITE   6%  4.4b  98% 1.6c   BOSS    1%  3.9b  99% 1.7c   </t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t xml:space="preserve">  NEWCOMER  FLOOR 1  EARLY 100%  2.4b  15% 1.2c   LATE  100%  4.0b  34% 1.8c   ELITE  98%  4.5b  41% 1.9c   BOSS   47%  6.9b  78% 1.8c   </t>
+          <t xml:space="preserve">  NEWCOMER  FLOOR 1  EARLY 100%  2.4b  16% 1.2c   LATE   99%  3.9b  35% 1.7c   ELITE  99%  4.5b  39% 1.9c   BOSS   42%  7.2b  84% 1.9c   </t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t xml:space="preserve">  NEWCOMER  FLOOR 2  EARLY  86%  5.1b  62% 1.9c   LATE   18%  4.4b  94% 1.5c   ELITE   8%  4.6b  97% 1.7c   BOSS    0%  4.5b  99% 1.6c   </t>
+          <t xml:space="preserve">  NEWCOMER  FLOOR 2  EARLY  90%  5.3b  62% 1.9c   LATE   11%  4.1b  96% 1.5c   ELITE   9%  4.8b  97% 1.8c   BOSS    0%  4.2b  99% 1.7c   </t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t xml:space="preserve">  NEWCOMER  FLOOR 3  EARLY   2%  3.3b  98% 1.4c   LATE    0%  2.1b 100% 1.0c   ELITE   0%  2.4b 100% 1.2c   BOSS    0%  2.3b 100% 1.1c   </t>
+          <t xml:space="preserve">  NEWCOMER  FLOOR 3  EARLY   4%  3.5b  99% 1.4c   LATE    0%  2.2b 100% 1.0c   ELITE   0%  2.4b 100% 1.2c   BOSS    0%  2.3b 100% 1.2c   </t>
         </is>
       </c>
     </row>
@@ -1614,251 +1614,272 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>EACH ENEMY leading its pack (normal floor 2 late, elite floor 2, boss floor 3), AVERAGE player : WIN PERCENT / BARS</t>
+          <t>EACH ENEMY leading its pack (normal floor 2 late, elite floor 2, boss floor 3) : WIN PERCENT / BARS  AVERAGE, then STRONG</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t xml:space="preserve">  HUSH                   77%  5.2b</t>
+          <t xml:space="preserve">  HUSH                   80%  5.1b    100%  4.0b    </t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t xml:space="preserve">  DEAD AIR               74%  5.1b</t>
+          <t xml:space="preserve">  DEAD AIR               74%  5.1b     99%  4.0b    </t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t xml:space="preserve">  THE LULL               79%  5.5b</t>
+          <t xml:space="preserve">  THE LULL               81%  5.7b    100%  4.2b    </t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t xml:space="preserve">  STATIC                 79%  5.1b</t>
+          <t xml:space="preserve">  STATIC                 78%  5.4b    100%  4.0b    </t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t xml:space="preserve">  THE MUTE CHOIR         72%  6.1b</t>
+          <t xml:space="preserve">  THE MUTE CHOIR         70%  6.1b     99%  4.7b    </t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t xml:space="preserve">  WHITE NOISE            47%  5.7b</t>
+          <t xml:space="preserve">  WHITE NOISE            40%  5.5b    100%  5.0b    </t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t xml:space="preserve">  REQUIEM                 0%  3.8b</t>
+          <t xml:space="preserve">  REQUIEM                 0%  4.2b     50%  8.4b    </t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t xml:space="preserve">  THE NAMELESS MASTER     1%  5.2b</t>
+          <t xml:space="preserve">  THE NAMELESS MASTER     2%  5.1b     92%  8.6b    </t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t xml:space="preserve">  THE DEVIL'S STRING      0%  3.6b</t>
+          <t xml:space="preserve">  THE DEVIL'S STRING      0%  3.5b     30%  8.1b    </t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t xml:space="preserve">  ROOM TONE              81%  5.5b</t>
+          <t xml:space="preserve">  ROOM TONE              84%  5.4b    100%  4.1b    </t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t xml:space="preserve">  THE CUE                87%  5.3b</t>
+          <t xml:space="preserve">  THE CUE                85%  5.3b    100%  4.1b    </t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t xml:space="preserve">  THE DAMPER             68%  5.5b</t>
+          <t xml:space="preserve">  THE DAMPER             64%  5.4b    100%  4.4b    </t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t xml:space="preserve">  STUTTER                85%  5.2b</t>
+          <t xml:space="preserve">  STUTTER                85%  5.0b    100%  3.9b    </t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t xml:space="preserve">  THE ROUND              68%  6.2b</t>
-        </is>
-      </c>
-    </row>
-    <row r="37"/>
+          <t xml:space="preserve">  THE ROUND              68%  6.3b    100%  4.7b    </t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  THE DEAF CROWN          0%  3.8b     62%  8.8b    </t>
+        </is>
+      </c>
+    </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>RUNS (3 floors, life carried over, no motifs) : WIN PERCENT  /  LOST ON FLOOR 1, 2, 3</t>
+          <t xml:space="preserve">  THE STAFF               0%  4.1b     44%  8.6b    </t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t xml:space="preserve">  NORMAL</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    FLAWLESS 100%    0% / 0% / 0%</t>
-        </is>
-      </c>
-    </row>
+          <t xml:space="preserve">  THE BLIND CANTOR        0%  4.2b     57%  8.4b    </t>
+        </is>
+      </c>
+    </row>
+    <row r="40"/>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t xml:space="preserve">    EXPERT   100%    0% / 0% / 0%</t>
+          <t>RUNS (3 floors, life carried over, no motifs) : WIN PERCENT  /  LOST ON FLOOR 1, 2, 3</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t xml:space="preserve">    STRONG    50%    0% / 10% / 38%</t>
+          <t xml:space="preserve">  NORMAL</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t xml:space="preserve">    AVERAGE    0%    30% / 68% / 0%</t>
+          <t xml:space="preserve">    FLAWLESS 100%    0% / 0% / 0%</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t xml:space="preserve">    NEWCOMER   0%    80% / 19% / 0%</t>
+          <t xml:space="preserve">    EXPERT    99%    0% / 0% / 0%</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t xml:space="preserve">  MAESTRO</t>
+          <t xml:space="preserve">    STRONG    61%    0% / 10% / 27%</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t xml:space="preserve">    FLAWLESS 100%    0% / 0% / 0%</t>
+          <t xml:space="preserve">    AVERAGE    0%    31% / 68% / 0%</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t xml:space="preserve">    EXPERT    79%    0% / 3% / 17%</t>
+          <t xml:space="preserve">    NEWCOMER   0%    88% / 12% / 0%</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t xml:space="preserve">    STRONG     0%    15% / 72% / 12%</t>
+          <t xml:space="preserve">  MAESTRO</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t xml:space="preserve">    AVERAGE    0%    94% / 5% / 0%</t>
+          <t xml:space="preserve">    FLAWLESS 100%    0% / 0% / 0%</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t xml:space="preserve">    NEWCOMER   0%    100% / 0% / 0%</t>
-        </is>
-      </c>
-    </row>
-    <row r="51"/>
+          <t xml:space="preserve">    EXPERT    76%    0% / 4% / 20%</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    STRONG     0%    15% / 73% / 11%</t>
+        </is>
+      </c>
+    </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>CONDUCTORS (runs as above, NORMAL) : WIN PERCENT  STRONG / AVERAGE</t>
+          <t xml:space="preserve">    AVERAGE    0%    94% / 5% / 0%</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t xml:space="preserve">  THE UNHEARING       58% / 0%</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  THE SHADOWLESS      51% / 0%</t>
-        </is>
-      </c>
-    </row>
+          <t xml:space="preserve">    NEWCOMER   0%    100% / 0% / 0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="54"/>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t xml:space="preserve">  THE METRONOME       51% / 0%</t>
+          <t>CONDUCTORS (runs as above, NORMAL) : WIN PERCENT  STRONG / AVERAGE</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t xml:space="preserve">  THE HEARTLESS       65% / 0%</t>
+          <t xml:space="preserve">  THE UNHEARING       52% / 0%</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t xml:space="preserve">  THE KING'S BATON    63% / 0%</t>
+          <t xml:space="preserve">  THE SHADOWLESS      52% / 0%</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t xml:space="preserve">  THE UNSIGNED        50% / 0%</t>
-        </is>
-      </c>
-    </row>
-    <row r="59"/>
+          <t xml:space="preserve">  THE METRONOME       47% / 0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  THE HEARTLESS       52% / 0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  THE KING'S BATON    60% / 0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  THE UNSIGNED        49% / 0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="62"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -8647,7 +8668,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D140"/>
+  <dimension ref="A1:D145"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" style="33" min="1" max="1"/>
@@ -9467,565 +9488,590 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>PRACTICE</t>
+          <t>Bosses of step 14</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>TurnPracticeHp</t>
+          <t>TurnByTouchMost</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>160</t>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>THE BLIND CANTOR : missed notes that come back in its next attack, at most</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>PRACTICE</t>
+          <t>Bosses of step 14</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>TurnPracticeSpeed</t>
+          <t>TurnCourtKeep</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>THE STAFF : the share of the band's damage it takes while another enemy stands</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>PRACTICE</t>
+          <t>Bosses of step 14</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>TurnPracticePower</t>
+          <t>TurnStaffEvery</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>each note hits this x TurnNoteDamage (4 life)</t>
+          <t>every this many attacks it strikes the floor (instead of a CADENZA)</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Enemy Attack</t>
+          <t>Bosses of step 14</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>TurnNotesMin</t>
+          <t>TurnStaffPower</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>{ 1, 2, 3 }</t>
+          <t>1.5</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>ELITE and BOSS</t>
+          <t>that one note hits everyone this much harder</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Enemy Attack</t>
+          <t>Bosses of step 14</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>TurnNotesMax</t>
+          <t>TurnThorns</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>{ 2, 3, 4 }</t>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>THE DEAF CROWN : life lost by a musician who breaks the DECREE (x the floor's note scale)</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Enemy Attack</t>
+          <t>PRACTICE</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>TurnSmallNotesMin</t>
+          <t>TurnPracticeHp</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>{ 1, 1, 2 }</t>
-        </is>
-      </c>
-      <c r="D45" t="inlineStr">
-        <is>
-          <t>ordinary enemies</t>
+          <t>160</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Enemy Attack</t>
+          <t>PRACTICE</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>TurnSmallNotesMax</t>
+          <t>TurnPracticeSpeed</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>{ 2, 2, 2 }</t>
+          <t>4</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Enemy Attack</t>
+          <t>PRACTICE</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>TurnNoteDamage</t>
+          <t>TurnPracticePower</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>2.2</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>step 12 : was 1.5, the user found NORMAL far too easy (turnsim STRONG 81 -&gt; 57 percent)</t>
+          <t>each note hits this x TurnNoteDamage (4 life)</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>PARRY</t>
+          <t>Enemy Attack</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>TurnParryGoodKeep</t>
+          <t>TurnNotesMin</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>0.5</t>
+          <t>{ 1, 2, 3 }</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>ELITE and BOSS</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>BREATH</t>
+          <t>Enemy Attack</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>TurnBreathMax</t>
+          <t>TurnNotesMax</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>{ 2, 3, 4 }</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>BREATH</t>
+          <t>Enemy Attack</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>TurnBreathStart</t>
+          <t>TurnSmallNotesMin</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>{ 1, 1, 2 }</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>ordinary enemies</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>BREATH</t>
+          <t>Enemy Attack</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>TurnBreathPerAttack</t>
+          <t>TurnSmallNotesMax</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>{ 2, 2, 2 }</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>BREATH</t>
+          <t>Enemy Attack</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>TurnBreathPerParry</t>
+          <t>TurnNoteDamage</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2.2</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>for each note parried PERFECT</t>
+          <t>step 12 : was 1.5, the user found NORMAL far too easy (turnsim STRONG 81 -&gt; 57 percent)</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>KNOCKED OUT</t>
+          <t>PARRY</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>TurnReviveHp</t>
+          <t>TurnParryGoodKeep</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0.5</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>OFF-BEAT</t>
+          <t>BREATH</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>TurnOffBeatMax</t>
+          <t>TurnBreathMax</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>10</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>OFF-BEAT</t>
+          <t>BREATH</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>TurnParryOffBeat</t>
+          <t>TurnBreathStart</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="D55" t="inlineStr">
-        <is>
-          <t>each note parried PERFECT</t>
+          <t>3</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>OFF-BEAT</t>
+          <t>BREATH</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>TurnOffBeatScale</t>
+          <t>TurnBreathPerAttack</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>1.5</t>
-        </is>
-      </c>
-      <c r="D56" t="inlineStr">
-        <is>
-          <t>damage against an enemy off the beat</t>
+          <t>1</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Statuses</t>
+          <t>BREATH</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>TurnDissonanceMost</t>
+          <t>TurnBreathPerParry</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>DISSONANCE stacks no higher</t>
+          <t>for each note parried PERFECT</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Statuses</t>
+          <t>KNOCKED OUT</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>TurnCrescendoStep</t>
+          <t>TurnReviveHp</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>0.15</t>
-        </is>
-      </c>
-      <c r="D58" t="inlineStr">
-        <is>
-          <t>CRESCENDO : each stack hits this much harder</t>
+          <t>1</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Statuses</t>
+          <t>OFF-BEAT</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>TurnCrescendoMost</t>
+          <t>TurnOffBeatMax</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>100</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Statuses</t>
+          <t>OFF-BEAT</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>TurnMuteTurns</t>
+          <t>TurnParryOffBeat</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>10</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>MUTE : turns without skills</t>
+          <t>each note parried PERFECT</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Statuses</t>
+          <t>OFF-BEAT</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>TurnGuardKeep</t>
+          <t>TurnOffBeatScale</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>0.5</t>
+          <t>1.5</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>GUARD : the share of a hit that gets through</t>
+          <t>damage against an enemy off the beat</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>COUNTER and CADENZA</t>
+          <t>Statuses</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>TurnCounterScale</t>
+          <t>TurnDissonanceMost</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>9</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>x the target's attack damage</t>
+          <t>DISSONANCE stacks no higher</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>COUNTER and CADENZA</t>
+          <t>Statuses</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>TurnCadenzaCounter</t>
+          <t>TurnCrescendoStep</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0.15</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>CRESCENDO : each stack hits this much harder</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>COUNTER and CADENZA</t>
+          <t>Statuses</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>TurnCadenzaEvery</t>
+          <t>TurnCrescendoMost</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>5</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>COUNTER and CADENZA</t>
+          <t>Statuses</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>TurnCadenzaPower</t>
+          <t>TurnMuteTurns</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>1.5</t>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>MUTE : turns without skills</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Skill Notes</t>
+          <t>Statuses</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>TurnHoldBase</t>
+          <t>TurnGuardKeep</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>0.6</t>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>GUARD : the share of a hit that gets through</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Skill Notes</t>
+          <t>COUNTER and CADENZA</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>TurnHoldGain</t>
+          <t>TurnCounterScale</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>0.8</t>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>x the target's attack damage</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Skill Notes</t>
+          <t>COUNTER and CADENZA</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>TurnRollPerfect</t>
+          <t>TurnCadenzaCounter</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Skill Notes</t>
+          <t>COUNTER and CADENZA</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>TurnRollGood</t>
+          <t>TurnCadenzaEvery</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
@@ -10037,17 +10083,17 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Skill Notes</t>
+          <t>COUNTER and CADENZA</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>MaestroTurnRollPerfect</t>
+          <t>TurnCadenzaPower</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>1.5</t>
         </is>
       </c>
     </row>
@@ -10059,227 +10105,202 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>MaestroTurnRollGood</t>
+          <t>TurnHoldBase</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>0.6</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Conductors</t>
+          <t>Skill Notes</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>TurnSignatureNeed</t>
+          <t>TurnHoldGain</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>0.8</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Conductors</t>
+          <t>Skill Notes</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>TurnBeethovenMost</t>
+          <t>TurnRollPerfect</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>0.5</t>
-        </is>
-      </c>
-      <c r="D73" t="inlineStr">
-        <is>
-          <t>THE UNHEARING's PASSIVE : up to this much harder as the band's life runs out</t>
+          <t>5</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Conductors</t>
+          <t>Skill Notes</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>TurnBoltDamage</t>
+          <t>TurnRollGood</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>14</t>
-        </is>
-      </c>
-      <c r="D74" t="inlineStr">
-        <is>
-          <t>LIGHTNING : damage to every enemy at full strength (x1)</t>
+          <t>3</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Conductors</t>
+          <t>Skill Notes</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>TurnMozartRun</t>
+          <t>MaestroTurnRollPerfect</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="D75" t="inlineStr">
-        <is>
-          <t>THE SHADOWLESS's PASSIVE : this many PERFECTs in a row give 1 breath</t>
+          <t>6</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Conductors</t>
+          <t>Skill Notes</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>TurnFeatherPerStroke</t>
+          <t>MaestroTurnRollGood</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="D76" t="inlineStr">
-        <is>
-          <t>FEATHER : free ATTACKs per stroke that lands (step 12, was 1 extra turn : 25 percent of STRONG runs won)</t>
+          <t>4</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>The other four of the lore</t>
+          <t>Conductors</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>TurnFugueScale</t>
+          <t>TurnSignatureNeed</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>1.8</t>
-        </is>
-      </c>
-      <c r="D77" t="inlineStr">
-        <is>
-          <t>FUGUE : the echo plays at the SIGNATURE's strength x this (step 13 : was 1, THE METRONOME was the weakest at 44 percent)</t>
+          <t>6</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>The other four of the lore</t>
+          <t>Conductors</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>TurnPaganiniLife</t>
+          <t>TurnBeethovenMost</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>0.5</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>THE HEARTLESS's PASSIVE : life paid for each BREATH a skill is short of</t>
+          <t>THE UNHEARING's PASSIVE : up to this much harder as the band's life runs out</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>The other four of the lore</t>
+          <t>Conductors</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>TurnCapricePrice</t>
+          <t>TurnBoltDamage</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>0.2</t>
+          <t>14</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>CAPRICE : when it ends, every musician pays this share of their life (never below 1, step 13 : was 0.1)</t>
+          <t>LIGHTNING : damage to every enemy at full strength (x1)</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>The other four of the lore</t>
+          <t>Conductors</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>TurnCapricePerStroke</t>
+          <t>TurnMozartRun</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>CAPRICE : turns per stroke that lands (step 12, a bar has more turns now)</t>
+          <t>THE SHADOWLESS's PASSIVE : this many PERFECTs in a row give 1 breath</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>The other four of the lore</t>
+          <t>Conductors</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>TurnLullyWindow</t>
+          <t>TurnFeatherPerStroke</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>0.01</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>THE KING'S BATON's PASSIVE : seconds added to both parry windows (0.05 won 99 percent of STRONG runs, the others 83 to 90;</t>
+          <t>FEATHER : free ATTACKs per stroke that lands (step 12, was 1 extra turn : 25 percent of STRONG runs won)</t>
         </is>
       </c>
     </row>
@@ -10291,17 +10312,17 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>TurnSunHeal</t>
+          <t>TurnFugueScale</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>1.8</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>THE SUN : life back for every musician at full strength (step 13 : was 12, THE KING'S BATON was the strongest at 71 percent)</t>
+          <t>FUGUE : the echo plays at the SIGNATURE's strength x this (step 13 : was 1, THE METRONOME was the weakest at 44 percent)</t>
         </is>
       </c>
     </row>
@@ -10313,17 +10334,17 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>TurnFannyScale</t>
+          <t>TurnPaganiniLife</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>0.25</t>
+          <t>3</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>THE UNSIGNED's PASSIVE : FANNY's voice hits this much harder</t>
+          <t>THE HEARTLESS's PASSIVE : life paid for each BREATH a skill is short of</t>
         </is>
       </c>
     </row>
@@ -10335,17 +10356,17 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>TurnFelixHeal</t>
+          <t>TurnCapricePrice</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>1.5</t>
+          <t>0.2</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>FELIX's voice heals this much more</t>
+          <t>CAPRICE : when it ends, every musician pays this share of their life (never below 1, step 13 : was 0.1)</t>
         </is>
       </c>
     </row>
@@ -10357,17 +10378,17 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>TurnFelixCrescendo</t>
+          <t>TurnCapricePerStroke</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>and gives this much more CRESCENDO</t>
+          <t>CAPRICE : turns per stroke that lands (step 12, a bar has more turns now)</t>
         </is>
       </c>
     </row>
@@ -10379,17 +10400,17 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>TurnDuetDamage</t>
+          <t>TurnLullyWindow</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>0.01</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>TWO VOICES : damage to every enemy at full strength (step 13 : was 9 and 6, THE UNSIGNED 46 percent)</t>
+          <t>THE KING'S BATON's PASSIVE : seconds added to both parry windows (0.05 won 99 percent of STRONG runs, the others 83 to 90;</t>
         </is>
       </c>
     </row>
@@ -10401,7 +10422,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>TurnDuetHeal</t>
+          <t>TurnSunHeal</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
@@ -10411,41 +10432,41 @@
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>and life back for every musician</t>
+          <t>THE SUN : life back for every musician at full strength (step 13 : was 12, THE KING'S BATON was the strongest at 71 percent)</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>Musician Traits in the turn battle</t>
+          <t>The other four of the lore</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>TurnCountsWindow</t>
+          <t>TurnFannyScale</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>0.05</t>
+          <t>0.25</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>COUNTS ALOUD (ANNA) : seconds added to her PERFECT window</t>
+          <t>THE UNSIGNED's PASSIVE : FANNY's voice hits this much harder</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>Musician Traits in the turn battle</t>
+          <t>The other four of the lore</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>TurnQuietScale</t>
+          <t>TurnFelixHeal</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
@@ -10455,73 +10476,73 @@
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>THE QUIET PART (KLARA) : against an enemy showing a p note</t>
+          <t>FELIX's voice heals this much more</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>Musician Traits in the turn battle</t>
+          <t>The other four of the lore</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>TurnMomentumMost</t>
+          <t>TurnFelixCrescendo</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>MOMENTUM (OTTO) : power gained by hits in a row, at most</t>
+          <t>and gives this much more CRESCENDO</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>Musician Traits in the turn battle</t>
+          <t>The other four of the lore</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>TurnByEarScale</t>
+          <t>TurnDuetDamage</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>1.5</t>
+          <t>12</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>BY EAR (MALI) : against an enemy that is OFF-BEAT</t>
+          <t>TWO VOICES : damage to every enemy at full strength (step 13 : was 9 and 6, THE UNSIGNED 46 percent)</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>Musician Traits in the turn battle</t>
+          <t>The other four of the lore</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>TurnHeldNoteShare</t>
+          <t>TurnDuetHeal</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>0.4</t>
+          <t>8</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>HELD NOTE (CHAI) : his ATTACK hits again for this share</t>
+          <t>and life back for every musician</t>
         </is>
       </c>
     </row>
@@ -10533,17 +10554,17 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>TurnStepBetterScale</t>
+          <t>TurnCountsWindow</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>1.3</t>
+          <t>0.05</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>ONE STEP BETTER (NUAN) : against an enemy showing an f note</t>
+          <t>COUNTS ALOUD (ANNA) : seconds added to her PERFECT window</t>
         </is>
       </c>
     </row>
@@ -10555,17 +10576,17 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>TurnFourBarsEvery</t>
+          <t>TurnQuietScale</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1.5</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>FOUR BARS STRAIGHT (LUKA) : every this many ATTACKs</t>
+          <t>THE QUIET PART (KLARA) : against an enemy showing a p note</t>
         </is>
       </c>
     </row>
@@ -10577,17 +10598,17 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>TurnFourBarsScale</t>
+          <t>TurnMomentumMost</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>hits this much harder</t>
+          <t>MOMENTUM (OTTO) : power gained by hits in a row, at most</t>
         </is>
       </c>
     </row>
@@ -10599,17 +10620,17 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>TurnLateBonus</t>
+          <t>TurnByEarScale</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>0.12</t>
+          <t>1.5</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>FASHIONABLY LATE (IRIS) : seconds after the GOOD window a late stroke still counts</t>
+          <t>BY EAR (MALI) : against an enemy that is OFF-BEAT</t>
         </is>
       </c>
     </row>
@@ -10621,117 +10642,117 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>TurnThunderSoften</t>
+          <t>TurnHeldNoteShare</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0.4</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>THE WHOLE FLOOR (BORIS) : taken off each note of the enemy's next attack</t>
+          <t>HELD NOTE (CHAI) : his ATTACK hits again for this share</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>ARCHIVE</t>
+          <t>Musician Traits in the turn battle</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>EchoesPerWin</t>
+          <t>TurnStepBetterScale</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1.3</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>each fight won</t>
+          <t>ONE STEP BETTER (NUAN) : against an enemy showing an f note</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>ARCHIVE</t>
+          <t>Musician Traits in the turn battle</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>EchoesPerFloor</t>
+          <t>TurnFourBarsEvery</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>4</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>each floor cleared</t>
+          <t>FOUR BARS STRAIGHT (LUKA) : every this many ATTACKs</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>ARCHIVE</t>
+          <t>Musician Traits in the turn battle</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>EchoesRunWon</t>
+          <t>TurnFourBarsScale</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>the whole run won</t>
+          <t>hits this much harder</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>ARCHIVE</t>
+          <t>Musician Traits in the turn battle</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>EchoesMaestro</t>
+          <t>TurnLateBonus</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>1.5</t>
+          <t>0.12</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>MAESTRO pays more</t>
+          <t>FASHIONABLY LATE (IRIS) : seconds after the GOOD window a late stroke still counts</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>ARCHIVE</t>
+          <t>Musician Traits in the turn battle</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>ArchiveLifePerLevel</t>
+          <t>TurnThunderSoften</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
@@ -10741,7 +10762,7 @@
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>STRONGER BAND</t>
+          <t>THE WHOLE FLOOR (BORIS) : taken off each note of the enemy's next attack</t>
         </is>
       </c>
     </row>
@@ -10753,17 +10774,17 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>ArchiveBreathPerLevel</t>
+          <t>EchoesPerWin</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>DEEP BREATH</t>
+          <t>each fight won</t>
         </is>
       </c>
     </row>
@@ -10775,17 +10796,17 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>ArchiveSignaturePerLevel</t>
+          <t>EchoesPerFloor</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>10</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>WARM UP</t>
+          <t>each floor cleared</t>
         </is>
       </c>
     </row>
@@ -10797,17 +10818,17 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>ArchiveShardsPerLevel</t>
+          <t>EchoesRunWon</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>25</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>SAVINGS</t>
+          <t>the whole run won</t>
         </is>
       </c>
     </row>
@@ -10819,127 +10840,127 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>ArchiveStagePerLevel</t>
+          <t>EchoesMaestro</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>1.5</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>FULL STAGE : musicians more on the field at the start (step 12)</t>
+          <t>MAESTRO pays more</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>Turn Motifs</t>
+          <t>ARCHIVE</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>TurnReedCaseHeal</t>
+          <t>ArchiveLifePerLevel</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>1.5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>REED CASE : wind players' healing</t>
+          <t>STRONGER BAND</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>Turn Motifs</t>
+          <t>ARCHIVE</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>TurnSpareSticksOffBeat</t>
+          <t>ArchiveBreathPerLevel</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>1.5</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>SPARE STICKS : percussion skills' OFF-BEAT</t>
+          <t>DEEP BREATH</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>Turn Motifs</t>
+          <t>ARCHIVE</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>TurnPianissimoBreath</t>
+          <t>ArchiveSignaturePerLevel</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>PIANISSIMO : more breath for a p note parried PERFECT</t>
+          <t>WARM UP</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>Turn Motifs</t>
+          <t>ARCHIVE</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>TurnBreathMarkStart</t>
+          <t>ArchiveShardsPerLevel</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>20</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>BREATH MARK : more breath at the start of a fight</t>
+          <t>SAVINGS</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>Turn Motifs</t>
+          <t>ARCHIVE</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>TurnTuttiScale</t>
+          <t>ArchiveStagePerLevel</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>1.25</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>TUTTI : skills that reach everyone</t>
+          <t>FULL STAGE : musicians more on the field at the start (step 12)</t>
         </is>
       </c>
     </row>
@@ -10951,17 +10972,17 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>TurnRubatoMiss</t>
+          <t>TurnReedCaseHeal</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>0.6</t>
+          <t>1.5</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>RUBATO : a skill note you MISS still plays at this (step 12)</t>
+          <t>REED CASE : wind players' healing</t>
         </is>
       </c>
     </row>
@@ -10973,17 +10994,17 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>TurnCrescendoStart</t>
+          <t>TurnSpareSticksOffBeat</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>1.5</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>CRESCENDO : stacks on every musician at the start</t>
+          <t>SPARE STICKS : percussion skills' OFF-BEAT</t>
         </is>
       </c>
     </row>
@@ -10995,17 +11016,17 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>TurnSforzandoScale</t>
+          <t>TurnPianissimoBreath</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>1.3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>SFORZANDO : a PERFECT f note</t>
+          <t>PIANISSIMO : more breath for a p note parried PERFECT</t>
         </is>
       </c>
     </row>
@@ -11017,7 +11038,7 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>TurnOvertureScale</t>
+          <t>TurnBreathMarkStart</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
@@ -11027,7 +11048,7 @@
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>OVERTURE : the band's first hit of a fight</t>
+          <t>BREATH MARK : more breath at the start of a fight</t>
         </is>
       </c>
     </row>
@@ -11039,17 +11060,17 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>TurnCounterpointScale</t>
+          <t>TurnTuttiScale</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1.25</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>COUNTERPOINT : the COUNTER</t>
+          <t>TUTTI : skills that reach everyone</t>
         </is>
       </c>
     </row>
@@ -11061,17 +11082,17 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>TurnAccelerandoShakes</t>
+          <t>TurnRubatoMiss</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0.6</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>ACCELERANDO : each shake of a roll counts this many</t>
+          <t>RUBATO : a skill note you MISS still plays at this (step 12)</t>
         </is>
       </c>
     </row>
@@ -11083,17 +11104,17 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>TurnGraceTimes</t>
+          <t>TurnCrescendoStart</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>GRACE NOTE : a spark that lands does its skill this many times</t>
+          <t>CRESCENDO : stacks on every musician at the start</t>
         </is>
       </c>
     </row>
@@ -11105,17 +11126,17 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>TurnMarcatoOffBeat</t>
+          <t>TurnSforzandoScale</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1.3</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>MARCATO : a PERFECT attack's OFF-BEAT, times this</t>
+          <t>SFORZANDO : a PERFECT f note</t>
         </is>
       </c>
     </row>
@@ -11127,17 +11148,17 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>TurnConBrioNeed</t>
+          <t>TurnOvertureScale</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>CON BRIO : PERFECTs the SIGNATURE needs instead</t>
+          <t>OVERTURE : the band's first hit of a fight</t>
         </is>
       </c>
     </row>
@@ -11149,17 +11170,17 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>TurnCodaBelow</t>
+          <t>TurnCounterpointScale</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>0.25</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>CODA : an enemy under this share of its life</t>
+          <t>COUNTERPOINT : the COUNTER</t>
         </is>
       </c>
     </row>
@@ -11171,51 +11192,51 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>TurnCodaScale</t>
+          <t>TurnAccelerandoShakes</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>1.5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>takes this much more</t>
+          <t>ACCELERANDO : each shake of a roll counts this many</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>ONE BAR motifs</t>
+          <t>Turn Motifs</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>TurnDownbeatScale</t>
+          <t>TurnGraceTimes</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>1.5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>DOWNBEAT : the first move of a bar</t>
+          <t>GRACE NOTE : a spark that lands does its skill this many times</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>ONE BAR motifs</t>
+          <t>Turn Motifs</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>TurnEntranceScale</t>
+          <t>TurnMarcatoOffBeat</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
@@ -11225,161 +11246,161 @@
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>ENTRANCE : a called musician's moves in their first bar</t>
+          <t>MARCATO : a PERFECT attack's OFF-BEAT, times this</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>ONE BAR motifs</t>
+          <t>Turn Motifs</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>TurnGreenRoomHeal</t>
+          <t>TurnConBrioNeed</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>GREEN ROOM : life back for each musician on the BENCH at the end of a bar</t>
+          <t>CON BRIO : PERFECTs the SIGNATURE needs instead</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>ONE BAR motifs</t>
+          <t>Turn Motifs</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>TurnUnisonScale</t>
+          <t>TurnCodaBelow</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0.25</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>UNISON : the last ATTACK of a bar that all goes at one enemy</t>
+          <t>CODA : an enemy under this share of its life</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>Turn Feel</t>
+          <t>Turn Motifs</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>TurnRingTime</t>
+          <t>TurnCodaScale</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>1.1</t>
+          <t>1.5</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>from a note showing to the moment to swipe</t>
+          <t>takes this much more</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>Turn Feel</t>
+          <t>ONE BAR motifs</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>MaestroTurnRingTime</t>
+          <t>TurnDownbeatScale</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>0.8</t>
+          <t>1.5</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>MAESTRO</t>
+          <t>DOWNBEAT : the first move of a bar</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>Turn Feel</t>
+          <t>ONE BAR motifs</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>TurnNoteGap</t>
+          <t>TurnEntranceScale</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>0.55</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>between the notes of one enemy attack</t>
+          <t>ENTRANCE : a called musician's moves in their first bar</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>Turn Feel</t>
+          <t>ONE BAR motifs</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>TurnPause</t>
+          <t>TurnGreenRoomHeal</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>0.8</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>after a turn, before the next one starts</t>
+          <t>GREEN ROOM : life back for each musician on the BENCH at the end of a bar</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>Turn Feel</t>
+          <t>ONE BAR motifs</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>TurnHitStop</t>
+          <t>TurnUnisonScale</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>0.075</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>the band and TACET freeze for a moment on a PERFECT</t>
+          <t>UNISON : the last ATTACK of a bar that all goes at one enemy</t>
         </is>
       </c>
     </row>
@@ -11391,17 +11412,17 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>TurnStrikeTime</t>
+          <t>TurnRingTime</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>0.42</t>
+          <t>1.1</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>ONE BAR : how long an ATTACK's lunge takes, there and back</t>
+          <t>from a note showing to the moment to swipe</t>
         </is>
       </c>
     </row>
@@ -11413,17 +11434,17 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>TurnStrikeImpact</t>
+          <t>MaestroTurnRingTime</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>0.16</t>
+          <t>0.8</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>when in it the hit lands</t>
+          <t>MAESTRO</t>
         </is>
       </c>
     </row>
@@ -11435,17 +11456,17 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>TurnStrikeStop</t>
+          <t>TurnNoteGap</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>0.07</t>
+          <t>0.55</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>the freeze when it lands</t>
+          <t>between the notes of one enemy attack</t>
         </is>
       </c>
     </row>
@@ -11457,17 +11478,17 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>TurnKillStop</t>
+          <t>TurnPause</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>0.18</t>
+          <t>0.8</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>the freeze when an enemy falls silent</t>
+          <t>after a turn, before the next one starts</t>
         </is>
       </c>
     </row>
@@ -11479,17 +11500,17 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>TurnEndTime</t>
+          <t>TurnHitStop</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>2.2</t>
+          <t>0.075</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>the win or lose banner stays this long</t>
+          <t>the band and TACET freeze for a moment on a PERFECT</t>
         </is>
       </c>
     </row>
@@ -11501,17 +11522,17 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>TurnSparkGap</t>
+          <t>TurnStrikeTime</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>0.3</t>
+          <t>0.42</t>
         </is>
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>a spark comes this soon after the note before it</t>
+          <t>ONE BAR : how long an ATTACK's lunge takes, there and back</t>
         </is>
       </c>
     </row>
@@ -11523,17 +11544,17 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>TurnHoldTime</t>
+          <t>TurnStrikeImpact</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>0.8</t>
+          <t>0.16</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
         <is>
-          <t>how long a HOLD note wants holding</t>
+          <t>when in it the hit lands</t>
         </is>
       </c>
     </row>
@@ -11545,17 +11566,17 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>TurnHoldStill</t>
+          <t>TurnStrikeStop</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>0.07</t>
         </is>
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>pixels per second the baton may drift and still count as still</t>
+          <t>the freeze when it lands</t>
         </is>
       </c>
     </row>
@@ -11567,15 +11588,125 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
+          <t>TurnKillStop</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>0.18</t>
+        </is>
+      </c>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>the freeze when an enemy falls silent</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>Turn Feel</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>TurnEndTime</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>2.2</t>
+        </is>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>the win or lose banner stays this long</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>Turn Feel</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>TurnSparkGap</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>0.3</t>
+        </is>
+      </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>a spark comes this soon after the note before it</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>Turn Feel</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>TurnHoldTime</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>0.8</t>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>how long a HOLD note wants holding</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>Turn Feel</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>TurnHoldStill</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>260</t>
+        </is>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>pixels per second the baton may drift and still count as still</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>Turn Feel</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
           <t>TurnRollTime</t>
         </is>
       </c>
-      <c r="C140" t="inlineStr">
+      <c r="C145" t="inlineStr">
         <is>
           <t>1.2</t>
         </is>
       </c>
-      <c r="D140" t="inlineStr">
+      <c r="D145" t="inlineStr">
         <is>
           <t>how long a ROLL note lasts</t>
         </is>
@@ -11592,7 +11723,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I15"/>
+  <dimension ref="A1:I18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" style="33" min="1" max="1"/>
@@ -12250,6 +12381,133 @@
       </c>
       <c r="I15" t="inlineStr"/>
     </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>THE DEAF CROWN</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Boss</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>240</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>7</v>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Uf Uf Uf Df, Lf Rf Df</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>DECREE (1)</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Each bar it forbids SKILLS or ATTACKS, and breaking it hurts. It never takes a COUNTER.</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>THE STAFF</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Boss</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>250</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>6</v>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Df Dmf Df, Dmf Lmf Dmf Rmf</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>THE COURT (1)</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>While its court stands it takes half. Every third attack it strikes the floor and hits everyone.</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>THE BLIND CANTOR</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Boss</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>240</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="E18" t="n">
+        <v>6</v>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Df Umf Df Umf, Lmf Rmf Lp Rp</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>BY TOUCH (1)</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>It strikes the seats in turn, front to back. A note you miss comes back in its next attack.</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Alpha7 step 15: seats start the fight, longer fights, consistency fixes
- a run starts with 2 seats (FULL STAGE 3, EXTRA SEAT sold again); everyone
  seated on the BAND page starts the fight, the rest wait on the bench
- ATTACK x0.55 and 2 BREATH each, enemy life x1.6/2.1/2.7, notes 1.85:
  fights about 1.45x longer, ATTACK 68 -> 36 percent of the band's damage,
  run win rates unchanged in turnsim; HEARTLESS and THE SUN retuned
- twelve places where a page disagreed with the rules (shop motif text,
  Paganini numbers, life on musician cards, rest and route words, event
  life, BARS, tutorial and title tips, MUTE CHOIR, motif floors, CIRCULAR)
- turnsim prints the ATTACK/skill damage share; turncheck 113/113

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WqLsaY7gVTeQY89VfVgASG
</commit_message>
<xml_diff>
--- a/docs/TACET_Balance.xlsx
+++ b/docs/TACET_Balance.xlsx
@@ -1381,7 +1381,7 @@
       </c>
       <c r="G5" s="68" t="inlineStr">
         <is>
-          <t>The 4/4 shape : for two turns per stroke that lands, a MISS is GOOD and a GOOD is PERFECT. Then every musician pays 10 percent of their life.</t>
+          <t xml:space="preserve">The 4/4 shape : for two turns per stroke that lands, a MISS is GOOD and a GOOD is PERFECT. Then every musician pays </t>
         </is>
       </c>
     </row>
@@ -1470,7 +1470,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A62"/>
+  <dimension ref="A1:A63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="140" customWidth="1" style="33" min="1" max="1"/>
@@ -1508,378 +1508,385 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t xml:space="preserve">  FLAWLESS  FLOOR 1  EARLY 100%  2.0b   0% 1.8c   LATE  100%  2.9b   0% 2.0c   ELITE 100%  3.0b   0% 1.9c   BOSS  100%  5.0b   0% 2.0c   </t>
+          <t xml:space="preserve">  FLAWLESS  FLOOR 1  EARLY 100%  3.0b   0% 2.0c   LATE  100%  3.0b   0% 2.0c   ELITE 100%  4.0b   0% 2.0c   BOSS  100%  6.9b   0% 2.0c   </t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t xml:space="preserve">  FLAWLESS  FLOOR 2  EARLY 100%  3.0b   0% 2.0c   LATE  100%  3.2b   0% 2.0c   ELITE 100%  3.9b   0% 2.0c   BOSS  100%  5.9b   0% 2.0c   </t>
+          <t xml:space="preserve">  FLAWLESS  FLOOR 2  EARLY 100%  3.5b   0% 2.0c   LATE  100%  4.6b   0% 2.0c   ELITE 100%  5.1b   0% 2.0c   BOSS  100%  8.6b   0% 2.0c   </t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t xml:space="preserve">  FLAWLESS  FLOOR 3  EARLY 100%  3.8b   0% 2.0c   LATE  100%  4.2b   0% 2.0c   ELITE 100%  4.4b   0% 2.0c   BOSS  100%  7.0b   1% 2.0c   </t>
+          <t xml:space="preserve">  FLAWLESS  FLOOR 3  EARLY 100%  5.3b   0% 2.0c   LATE  100%  6.5b   0% 2.0c   ELITE 100%  7.0b   0% 2.0c   BOSS  100% 11.5b   0% 2.0c   </t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t xml:space="preserve">  EXPERT    FLOOR 1  EARLY 100%  2.1b   2% 1.5c   LATE  100%  3.0b   5% 2.0c   ELITE 100%  3.4b   5% 2.0c   BOSS  100%  5.1b  12% 2.0c   </t>
+          <t xml:space="preserve">  EXPERT    FLOOR 1  EARLY 100%  3.0b   3% 2.0c   LATE  100%  3.5b   5% 2.0c   ELITE 100%  4.2b   4% 2.0c   BOSS  100%  7.1b   8% 2.0c   </t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t xml:space="preserve">  EXPERT    FLOOR 2  EARLY 100%  3.2b   8% 1.9c   LATE  100%  3.6b  11% 2.0c   ELITE 100%  4.2b  14% 2.0c   BOSS  100%  6.2b  20% 2.0c   </t>
+          <t xml:space="preserve">  EXPERT    FLOOR 2  EARLY 100%  4.2b   8% 2.0c   LATE  100%  5.2b  11% 2.0c   ELITE 100%  5.7b  13% 2.0c   BOSS  100%  9.2b  19% 2.0c   </t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t xml:space="preserve">  EXPERT    FLOOR 3  EARLY 100%  4.0b  12% 2.0c   LATE  100%  4.8b  15% 2.0c   ELITE 100%  5.1b  19% 2.0c   BOSS  100%  7.7b  29% 2.0c   </t>
+          <t xml:space="preserve">  EXPERT    FLOOR 3  EARLY 100%  6.0b  12% 2.0c   LATE  100%  7.0b  15% 2.0c   ELITE 100%  8.0b  21% 2.0c   BOSS   98% 12.5b  31% 2.0c   </t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t xml:space="preserve">  STRONG    FLOOR 1  EARLY 100%  2.1b   5% 1.4c   LATE  100%  3.2b  11% 2.0c   ELITE 100%  3.7b  12% 1.9c   BOSS  100%  5.6b  25% 2.0c   </t>
+          <t xml:space="preserve">  STRONG    FLOOR 1  EARLY 100%  3.1b   6% 2.0c   LATE  100%  4.0b  13% 2.0c   ELITE 100%  4.7b  11% 2.0c   BOSS  100%  7.9b  22% 2.0c   </t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t xml:space="preserve">  STRONG    FLOOR 2  EARLY 100%  3.8b  18% 1.9c   LATE  100%  4.2b  23% 2.0c   ELITE 100%  4.8b  28% 2.0c   BOSS   91%  7.3b  51% 2.0c   </t>
+          <t xml:space="preserve">  STRONG    FLOOR 2  EARLY 100%  4.8b  16% 2.0c   LATE  100%  6.0b  21% 2.0c   ELITE 100%  6.9b  29% 2.0c   BOSS   85% 10.7b  50% 2.0c   </t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t xml:space="preserve">  STRONG    FLOOR 3  EARLY 100%  4.8b  28% 2.0c   LATE   98%  5.7b  40% 2.0c   ELITE  88%  6.5b  56% 2.0c   BOSS   53%  8.2b  78% 2.0c   </t>
+          <t xml:space="preserve">  STRONG    FLOOR 3  EARLY 100%  7.2b  26% 2.0c   LATE   99%  8.6b  35% 2.0c   ELITE  80%  9.7b  61% 2.0c   BOSS   32% 11.9b  86% 2.0c   </t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t xml:space="preserve">  AVERAGE   FLOOR 1  EARLY 100%  2.3b  10% 1.3c   LATE  100%  3.5b  22% 1.9c   ELITE 100%  4.1b  24% 1.9c   BOSS   87%  7.1b  62% 2.0c   </t>
+          <t xml:space="preserve">  AVERAGE   FLOOR 1  EARLY 100%  3.5b  11% 2.0c   LATE  100%  5.2b  24% 2.0c   ELITE 100%  6.0b  26% 2.0c   BOSS   74% 10.4b  63% 2.0c   </t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t xml:space="preserve">  AVERAGE   FLOOR 2  EARLY  98%  4.4b  39% 1.9c   LATE   78%  5.4b  67% 1.9c   ELITE  67%  5.9b  73% 1.9c   BOSS   13%  6.2b  95% 1.9c   </t>
+          <t xml:space="preserve">  AVERAGE   FLOOR 2  EARLY  96%  6.8b  43% 2.0c   LATE   68%  8.0b  71% 2.0c   ELITE  37%  8.4b  89% 2.0c   BOSS    7%  8.0b  96% 2.0c   </t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t xml:space="preserve">  AVERAGE   FLOOR 3  EARLY  52%  5.3b  80% 1.8c   LATE   17%  4.3b  93% 1.6c   ELITE   6%  4.4b  98% 1.6c   BOSS    1%  3.9b  99% 1.7c   </t>
+          <t xml:space="preserve">  AVERAGE   FLOOR 3  EARLY  38%  8.4b  86% 2.0c   LATE    3%  5.4b  98% 1.8c   ELITE   1%  5.4b  99% 1.9c   BOSS    0%  4.8b 100% 1.9c   </t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t xml:space="preserve">  NEWCOMER  FLOOR 1  EARLY 100%  2.4b  16% 1.2c   LATE   99%  3.9b  35% 1.7c   ELITE  99%  4.5b  39% 1.9c   BOSS   42%  7.2b  84% 1.9c   </t>
+          <t xml:space="preserve">  NEWCOMER  FLOOR 1  EARLY 100%  4.0b  18% 2.0c   LATE   98%  6.9b  46% 2.0c   ELITE  94%  8.1b  53% 2.0c   BOSS   19% 10.0b  92% 2.0c   </t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t xml:space="preserve">  NEWCOMER  FLOOR 2  EARLY  90%  5.3b  62% 1.9c   LATE   11%  4.1b  96% 1.5c   ELITE   9%  4.8b  97% 1.8c   BOSS    0%  4.2b  99% 1.7c   </t>
+          <t xml:space="preserve">  NEWCOMER  FLOOR 2  EARLY  54%  8.1b  79% 2.0c   LATE    1%  5.2b  99% 1.8c   ELITE   1%  5.6b  99% 1.9c   BOSS    0%  4.6b 100% 1.9c   </t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t xml:space="preserve">  NEWCOMER  FLOOR 3  EARLY   4%  3.5b  99% 1.4c   LATE    0%  2.2b 100% 1.0c   ELITE   0%  2.4b 100% 1.2c   BOSS    0%  2.3b 100% 1.2c   </t>
-        </is>
-      </c>
-    </row>
-    <row r="21"/>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>EACH ENEMY leading its pack (normal floor 2 late, elite floor 2, boss floor 3) : WIN PERCENT / BARS  AVERAGE, then STRONG</t>
-        </is>
-      </c>
-    </row>
+          <t xml:space="preserve">  NEWCOMER  FLOOR 3  EARLY   0%  4.2b 100% 1.8c   LATE    0%  2.8b 100% 1.5c   ELITE   0%  3.1b 100% 1.8c   BOSS    0%  2.9b 100% 1.6c   </t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  DAMAGE SHARE in all of the fights above : ATTACK 36%  SKILLS 63%</t>
+        </is>
+      </c>
+    </row>
+    <row r="22"/>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t xml:space="preserve">  HUSH                   80%  5.1b    100%  4.0b    </t>
+          <t>EACH ENEMY leading its pack (normal floor 2 late, elite floor 2, boss floor 3) : WIN PERCENT / BARS  AVERAGE, then STRONG</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t xml:space="preserve">  DEAD AIR               74%  5.1b     99%  4.0b    </t>
+          <t xml:space="preserve">  HUSH                   61%  7.7b    100%  6.0b    </t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t xml:space="preserve">  THE LULL               81%  5.7b    100%  4.2b    </t>
+          <t xml:space="preserve">  DEAD AIR               56%  7.7b    100%  6.0b    </t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t xml:space="preserve">  STATIC                 78%  5.4b    100%  4.0b    </t>
+          <t xml:space="preserve">  THE LULL               74%  8.8b    100%  6.3b    </t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t xml:space="preserve">  THE MUTE CHOIR         70%  6.1b     99%  4.7b    </t>
+          <t xml:space="preserve">  STATIC                 67%  8.0b    100%  5.9b    </t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t xml:space="preserve">  WHITE NOISE            40%  5.5b    100%  5.0b    </t>
+          <t xml:space="preserve">  THE MUTE CHOIR         50%  8.7b    100%  6.7b    </t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t xml:space="preserve">  REQUIEM                 0%  4.2b     50%  8.4b    </t>
+          <t xml:space="preserve">  WHITE NOISE            21%  7.6b     99%  7.2b    </t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t xml:space="preserve">  THE NAMELESS MASTER     2%  5.1b     92%  8.6b    </t>
+          <t xml:space="preserve">  REQUIEM                 0%  4.6b     25%  12.0b    </t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t xml:space="preserve">  THE DEVIL'S STRING      0%  3.5b     30%  8.1b    </t>
+          <t xml:space="preserve">  THE NAMELESS MASTER     0%  6.5b     81%  13.5b    </t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t xml:space="preserve">  ROOM TONE              84%  5.4b    100%  4.1b    </t>
+          <t xml:space="preserve">  THE DEVIL'S STRING      0%  4.1b      6%  10.3b    </t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t xml:space="preserve">  THE CUE                85%  5.3b    100%  4.1b    </t>
+          <t xml:space="preserve">  ROOM TONE              73%  8.2b    100%  6.2b    </t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t xml:space="preserve">  THE DAMPER             64%  5.4b    100%  4.4b    </t>
+          <t xml:space="preserve">  THE CUE                74%  8.2b    100%  6.0b    </t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t xml:space="preserve">  STUTTER                85%  5.0b    100%  3.9b    </t>
+          <t xml:space="preserve">  THE DAMPER             51%  7.8b    100%  6.4b    </t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t xml:space="preserve">  THE ROUND              68%  6.3b    100%  4.7b    </t>
+          <t xml:space="preserve">  STUTTER                75%  7.8b    100%  5.6b    </t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t xml:space="preserve">  THE DEAF CROWN          0%  3.8b     62%  8.8b    </t>
+          <t xml:space="preserve">  THE ROUND              43%  8.9b     99%  6.9b    </t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t xml:space="preserve">  THE STAFF               0%  4.1b     44%  8.6b    </t>
+          <t xml:space="preserve">  THE DEAF CROWN          0%  4.4b     20%  12.9b    </t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t xml:space="preserve">  THE BLIND CANTOR        0%  4.2b     57%  8.4b    </t>
-        </is>
-      </c>
-    </row>
-    <row r="40"/>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>RUNS (3 floors, life carried over, no motifs) : WIN PERCENT  /  LOST ON FLOOR 1, 2, 3</t>
-        </is>
-      </c>
-    </row>
+          <t xml:space="preserve">  THE STAFF               0%  4.4b     28%  11.6b    </t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  THE BLIND CANTOR        0%  4.5b     29%  11.3b    </t>
+        </is>
+      </c>
+    </row>
+    <row r="41"/>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t xml:space="preserve">  NORMAL</t>
+          <t>RUNS (3 floors, life carried over, no motifs) : WIN PERCENT  /  LOST ON FLOOR 1, 2, 3</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t xml:space="preserve">    FLAWLESS 100%    0% / 0% / 0%</t>
+          <t xml:space="preserve">  NORMAL</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t xml:space="preserve">    EXPERT    99%    0% / 0% / 0%</t>
+          <t xml:space="preserve">    FLAWLESS 100%    0% / 0% / 0%</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t xml:space="preserve">    STRONG    61%    0% / 10% / 27%</t>
+          <t xml:space="preserve">    EXPERT   100%    0% / 0% / 0%</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t xml:space="preserve">    AVERAGE    0%    31% / 68% / 0%</t>
+          <t xml:space="preserve">    STRONG    55%    2% / 5% / 37%</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t xml:space="preserve">    NEWCOMER   0%    88% / 12% / 0%</t>
+          <t xml:space="preserve">    AVERAGE    0%    57% / 43% / 0%</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t xml:space="preserve">  MAESTRO</t>
+          <t xml:space="preserve">    NEWCOMER   0%    98% / 1% / 0%</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t xml:space="preserve">    FLAWLESS 100%    0% / 0% / 0%</t>
+          <t xml:space="preserve">  MAESTRO</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t xml:space="preserve">    EXPERT    76%    0% / 4% / 20%</t>
+          <t xml:space="preserve">    FLAWLESS 100%    0% / 0% / 0%</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t xml:space="preserve">    STRONG     0%    15% / 73% / 11%</t>
+          <t xml:space="preserve">    EXPERT    73%    1% / 2% / 23%</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t xml:space="preserve">    AVERAGE    0%    94% / 5% / 0%</t>
+          <t xml:space="preserve">    STRONG     0%    28% / 64% / 7%</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
+          <t xml:space="preserve">    AVERAGE    0%    99% / 0% / 0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
           <t xml:space="preserve">    NEWCOMER   0%    100% / 0% / 0%</t>
         </is>
       </c>
     </row>
-    <row r="54"/>
-    <row r="55">
-      <c r="A55" t="inlineStr">
-        <is>
-          <t>CONDUCTORS (runs as above, NORMAL) : WIN PERCENT  STRONG / AVERAGE</t>
-        </is>
-      </c>
-    </row>
+    <row r="55"/>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t xml:space="preserve">  THE UNHEARING       52% / 0%</t>
+          <t>CONDUCTORS (runs as above, NORMAL) : WIN PERCENT  STRONG / AVERAGE</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t xml:space="preserve">  THE SHADOWLESS      52% / 0%</t>
+          <t xml:space="preserve">  THE UNHEARING       62% / 0%</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t xml:space="preserve">  THE METRONOME       47% / 0%</t>
+          <t xml:space="preserve">  THE SHADOWLESS      53% / 0%</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t xml:space="preserve">  THE HEARTLESS       52% / 0%</t>
+          <t xml:space="preserve">  THE METRONOME       52% / 0%</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t xml:space="preserve">  THE KING'S BATON    60% / 0%</t>
+          <t xml:space="preserve">  THE HEARTLESS       62% / 0%</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t xml:space="preserve">  THE UNSIGNED        49% / 0%</t>
-        </is>
-      </c>
-    </row>
-    <row r="62"/>
+          <t xml:space="preserve">  THE KING'S BATON    55% / 0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  THE UNSIGNED        54% / 0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="63"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -8936,12 +8943,12 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0.55</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>ATTACK : no swipe, it always hits at this</t>
+          <t>ATTACK : no swipe, it always hits at this (step 15 : was 1, the user found ATTACK far too strong and fights too short.</t>
         </is>
       </c>
     </row>
@@ -8985,7 +8992,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>musicians on the field when a fight starts (FULL STAGE in the ARCHIVE adds 1)</t>
+          <t>seats on stage a run starts with (FULL STAGE in the ARCHIVE adds 1, EXTRA SEAT in the shop 1 each).</t>
         </is>
       </c>
     </row>
@@ -9222,7 +9229,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>1.15</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -9266,7 +9273,12 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>{ 1, 1.3, 1.6 }</t>
+          <t>{ 1.6, 2.1, 2.7 }</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>step 15 : was 1 / 1.3 / 1.6, fights about 1.5 times longer (the user asked for longer fights)</t>
         </is>
       </c>
     </row>
@@ -9608,7 +9620,12 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>160</t>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>x TurnFloorLife on floor 1 (1.6) = 96, step 15 (was 160 with the floor at 1)</t>
         </is>
       </c>
     </row>
@@ -9742,12 +9759,12 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>2.2</t>
+          <t>1.85</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>step 12 : was 1.5, the user found NORMAL far too easy (turnsim STRONG 81 -&gt; 57 percent)</t>
+          <t>step 12 : was 1.5, the user found NORMAL far too easy (turnsim STRONG 81 -&gt; 57 percent).</t>
         </is>
       </c>
     </row>
@@ -9815,7 +9832,12 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>step 15 : was 1. A weaker ATTACK pays for the skills instead</t>
         </is>
       </c>
     </row>
@@ -10339,12 +10361,12 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>6</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>THE HEARTLESS's PASSIVE : life paid for each BREATH a skill is short of</t>
+          <t>THE HEARTLESS's PASSIVE : life paid for each BREATH a skill is short of (step 15 : was 3, skills carry the fight now)</t>
         </is>
       </c>
     </row>
@@ -10427,12 +10449,12 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>6</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>THE SUN : life back for every musician at full strength (step 13 : was 12, THE KING'S BATON was the strongest at 71 percent)</t>
+          <t>THE SUN : life back for every musician at full strength (step 13 : was 12, THE KING'S BATON was the strongest at 71 percent. Step 15 : 8 -&gt; 6)</t>
         </is>
       </c>
     </row>
@@ -11987,7 +12009,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>A note that gets through takes the target's skills away for a turn.</t>
+          <t>A note you miss takes the target's skills away for a turn.</t>
         </is>
       </c>
       <c r="I6" t="inlineStr"/>

</xml_diff>

<commit_message>
Beta1 : block 2 part 7, the SIGNATURE grows at each boss
LIGHTNING becomes STORM (a bolt more each level, the storm of the Pastoral),
FUGUE becomes THE ART OF FUGUE (the echo plays on a move more), DUET becomes
DAS JAHR (CRESCENDO 2 for the band, then strike and heal x1.5). The level is
the floor reached, so the save needs nothing new. The boss's result page names
what the SIGNATURE becomes. The three conductors now sit close (62.5 / 66.0 /
63.7 in turnsim), and TACET's floors 2 and 3 grew once more to keep the run as
hard as before PATH : 64.1 percent (63.8 before), MAESTRO EXPERT 82.2 (82.0),
every legend's bands within 4.5 percent. turncheck 137/137.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LkyThr8Ag8ofurL2payU71
</commit_message>
<xml_diff>
--- a/docs/TACET_Balance.xlsx
+++ b/docs/TACET_Balance.xlsx
@@ -2097,7 +2097,7 @@
       </c>
       <c r="G2" s="68" t="inlineStr">
         <is>
-          <t>The 4/4 shape : every musician's next move plays twice. Better strokes, louder echo.</t>
+          <t>The 4/4 shape : every musician's next move plays twice. Better strokes, louder echo. Grows at each boss.</t>
         </is>
       </c>
     </row>
@@ -2134,7 +2134,7 @@
       </c>
       <c r="G3" s="68" t="inlineStr">
         <is>
-          <t>The 4/4 shape : strikes every enemy and throws it OFF-BEAT. Better strokes, bigger strike.</t>
+          <t>The 4/4 shape : strikes every enemy and throws it OFF-BEAT. Better strokes, bigger strike. Grows at each boss.</t>
         </is>
       </c>
     </row>
@@ -2282,7 +2282,7 @@
       </c>
       <c r="G7" s="68" t="inlineStr">
         <is>
-          <t>The 4/4 shape : FANNY strikes every enemy while ??? heals every musician.</t>
+          <t>The 4/4 shape : FANNY strikes every enemy while ??? heals every musician. Grows at each boss.</t>
         </is>
       </c>
     </row>
@@ -2342,14 +2342,14 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t xml:space="preserve">  FLAWLESS  FLOOR 2  EARLY 100%  3.2b   9%   LATE  100%  4.9b  13%   ELITE 100%  5.7b  15%   BOSS  100% 10.6b  17%   </t>
+          <t xml:space="preserve">  FLAWLESS  FLOOR 2  EARLY 100%  3.0b   8%   LATE  100%  4.5b  11%   ELITE 100%  5.5b  15%   BOSS  100%  9.9b  17%   </t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t xml:space="preserve">  FLAWLESS  FLOOR 3  EARLY 100%  4.9b  13%   LATE  100%  6.1b  16%   ELITE 100%  6.7b  18%   BOSS  100% 12.2b  17%   </t>
+          <t xml:space="preserve">  FLAWLESS  FLOOR 3  EARLY 100%  4.1b  11%   LATE  100%  5.0b  14%   ELITE 100%  6.0b  16%   BOSS  100% 10.7b  16%   </t>
         </is>
       </c>
     </row>
@@ -2363,77 +2363,77 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t xml:space="preserve">  EXPERT    FLOOR 2  EARLY 100%  3.3b  12%   LATE  100%  4.4b  17%   ELITE 100%  4.8b  17%   BOSS  100%  8.1b  23%   </t>
+          <t xml:space="preserve">  EXPERT    FLOOR 2  EARLY 100%  3.2b  12%   LATE  100%  4.1b  16%   ELITE 100%  4.6b  17%   BOSS  100%  8.0b  22%   </t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t xml:space="preserve">  EXPERT    FLOOR 3  EARLY 100%  5.3b  19%   LATE  100%  6.9b  21%   ELITE 100%  7.9b  22%   BOSS   99% 14.5b  25%   </t>
+          <t xml:space="preserve">  EXPERT    FLOOR 3  EARLY 100%  4.7b  18%   LATE  100%  5.6b  22%   ELITE 100%  7.0b  23%   BOSS   99% 12.7b  25%   </t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t xml:space="preserve">  STRONG    FLOOR 1  EARLY 100%  1.3b   5%   LATE  100%  2.1b  10%   ELITE 100%  2.5b  10%   BOSS  100%  4.2b  16%   </t>
+          <t xml:space="preserve">  STRONG    FLOOR 1  EARLY 100%  1.3b   5%   LATE  100%  2.2b  10%   ELITE 100%  2.4b  11%   BOSS  100%  4.1b  17%   </t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t xml:space="preserve">  STRONG    FLOOR 2  EARLY 100%  3.7b  18%   LATE  100%  4.8b  22%   ELITE 100%  5.9b  25%   BOSS   95% 10.8b  35%   </t>
+          <t xml:space="preserve">  STRONG    FLOOR 2  EARLY 100%  3.5b  18%   LATE  100%  4.6b  22%   ELITE  99%  5.7b  23%   BOSS   96% 10.8b  38%   </t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t xml:space="preserve">  STRONG    FLOOR 3  EARLY 100%  6.7b  25%   LATE  100%  9.0b  27%   ELITE  93% 11.9b  36%   BOSS   61% 18.4b  66%   </t>
+          <t xml:space="preserve">  STRONG    FLOOR 3  EARLY 100%  5.9b  26%   LATE  100%  7.4b  27%   ELITE  95% 10.0b  37%   BOSS   73% 15.4b  54%   </t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t xml:space="preserve">  AVERAGE   FLOOR 1  EARLY 100%  1.7b   9%   LATE  100%  2.9b  19%   ELITE 100%  3.1b  20%   BOSS   99%  5.6b  35%   </t>
+          <t xml:space="preserve">  AVERAGE   FLOOR 1  EARLY 100%  1.8b   9%   LATE  100%  2.9b  18%   ELITE 100%  3.1b  20%   BOSS   98%  5.4b  34%   </t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t xml:space="preserve">  AVERAGE   FLOOR 2  EARLY 100%  5.1b  29%   LATE   96%  8.1b  41%   ELITE  76% 10.6b  59%   BOSS   21% 11.7b  90%   </t>
+          <t xml:space="preserve">  AVERAGE   FLOOR 2  EARLY  99%  5.3b  31%   LATE   96%  7.9b  41%   ELITE  77% 10.6b  58%   BOSS   22% 11.3b  89%   </t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t xml:space="preserve">  AVERAGE   FLOOR 3  EARLY  63% 11.3b  65%   LATE   31% 10.9b  84%   ELITE  10% 10.9b  95%   BOSS    0%  7.8b  99%   </t>
+          <t xml:space="preserve">  AVERAGE   FLOOR 3  EARLY  67%  9.5b  64%   LATE   38%  8.6b  84%   ELITE  13%  9.9b  94%   BOSS    0%  6.5b 100%   </t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t xml:space="preserve">  NEWCOMER  FLOOR 1  EARLY 100%  2.1b  14%   LATE  100%  3.8b  30%   ELITE 100%  4.1b  29%   BOSS   69%  8.0b  71%   </t>
+          <t xml:space="preserve">  NEWCOMER  FLOOR 1  EARLY 100%  2.1b  14%   LATE  100%  3.8b  29%   ELITE 100%  4.1b  30%   BOSS   65%  8.1b  72%   </t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t xml:space="preserve">  NEWCOMER  FLOOR 2  EARLY  83%  7.9b  59%   LATE   28%  8.7b  89%   ELITE   7%  9.4b  98%   BOSS    0%  6.3b 100%   </t>
+          <t xml:space="preserve">  NEWCOMER  FLOOR 2  EARLY  81%  8.5b  61%   LATE   29%  8.3b  89%   ELITE   5%  9.1b  98%   BOSS    0%  6.3b  99%   </t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t xml:space="preserve">  NEWCOMER  FLOOR 3  EARLY   1%  5.8b  99%   LATE    0%  4.2b 100%   ELITE   0%  4.2b 100%   BOSS    0%  3.7b 100%   </t>
+          <t xml:space="preserve">  NEWCOMER  FLOOR 3  EARLY   1%  5.5b  99%   LATE    0%  3.7b 100%   ELITE   0%  4.5b 100%   BOSS    0%  3.4b 100%   </t>
         </is>
       </c>
     </row>
@@ -2462,21 +2462,21 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t xml:space="preserve">  EXPERT    31 /  66 /   2 /   0   x1.65</t>
+          <t xml:space="preserve">  EXPERT    31 /  66 /   1 /   0   x1.65</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t xml:space="preserve">  STRONG     3 /  51 /  43 /   2   x1.40</t>
+          <t xml:space="preserve">  STRONG     3 /  49 /  44 /   2   x1.39</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t xml:space="preserve">  AVERAGE    0 /   4 /  64 /  30   x1.19</t>
+          <t xml:space="preserve">  AVERAGE    0 /   4 /  63 /  31   x1.18</t>
         </is>
       </c>
     </row>
@@ -2498,119 +2498,119 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t xml:space="preserve">  HUSH                   94%  8.1b    100%  5.0b    </t>
+          <t xml:space="preserve">  HUSH                   98%  7.1b    100%  4.8b    </t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t xml:space="preserve">  DEAD AIR               94%  7.7b    100%  5.1b    </t>
+          <t xml:space="preserve">  DEAD AIR               96%  7.2b    100%  4.7b    </t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t xml:space="preserve">  THE LULL               96%  8.4b    100%  5.1b    </t>
+          <t xml:space="preserve">  THE LULL               97%  7.8b    100%  4.9b    </t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t xml:space="preserve">  STATIC                 92%  7.9b    100%  5.1b    </t>
+          <t xml:space="preserve">  STATIC                 92%  7.3b    100%  4.6b    </t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t xml:space="preserve">  THE MUTE CHOIR         89%  11.0b    100%  5.9b    </t>
+          <t xml:space="preserve">  THE MUTE CHOIR         93%  10.1b    100%  5.9b    </t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t xml:space="preserve">  WHITE NOISE            62%  8.8b    100%  5.6b    </t>
+          <t xml:space="preserve">  WHITE NOISE            66%  8.5b    100%  5.4b    </t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t xml:space="preserve">  REQUIEM                 0%  7.2b     52%  17.7b    </t>
+          <t xml:space="preserve">  REQUIEM                 0%  7.1b     67%  16.1b    </t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t xml:space="preserve">  THE NAMELESS MASTER     2%  11.3b     91%  17.3b    </t>
+          <t xml:space="preserve">  THE NAMELESS MASTER     3%  10.6b     94%  14.6b    </t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t xml:space="preserve">  THE DEVIL'S STRING      0%  6.4b     35%  16.8b    </t>
+          <t xml:space="preserve">  THE DEVIL'S STRING      0%  5.6b     43%  15.2b    </t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t xml:space="preserve">  ROOM TONE              94%  7.9b    100%  5.0b    </t>
+          <t xml:space="preserve">  ROOM TONE              97%  7.5b    100%  4.9b    </t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  THE CUE                97%  8.2b    100%  5.3b    </t>
+          <t xml:space="preserve">  THE CUE                96%  7.8b    100%  4.9b    </t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t xml:space="preserve">  THE DAMPER             96%  8.1b    100%  5.1b    </t>
+          <t xml:space="preserve">  THE DAMPER             94%  7.7b    100%  4.8b    </t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t xml:space="preserve">  STUTTER                98%  7.4b    100%  5.0b    </t>
+          <t xml:space="preserve">  STUTTER                99%  7.0b    100%  4.4b    </t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t xml:space="preserve">  THE ROUND              82%  12.9b    100%  5.9b    </t>
+          <t xml:space="preserve">  THE ROUND              76%  12.4b    100%  6.0b    </t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t xml:space="preserve">  THE DEAF CROWN          0%  5.7b     48%  21.1b    </t>
+          <t xml:space="preserve">  THE DEAF CROWN          0%  5.8b     61%  19.6b    </t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t xml:space="preserve">  THE STAFF               0%  7.9b     66%  18.7b    </t>
+          <t xml:space="preserve">  THE STAFF               0%  7.0b     73%  17.3b    </t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t xml:space="preserve">  THE BLIND CANTOR        0%  6.5b     62%  17.6b    </t>
+          <t xml:space="preserve">  THE BLIND CANTOR        0%  6.7b     77%  15.4b    </t>
         </is>
       </c>
     </row>
@@ -2632,35 +2632,35 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t xml:space="preserve">    FLAWLESS 100%    0% / 0% / 0%    2.8 / 4.4 / 5.1</t>
+          <t xml:space="preserve">    FLAWLESS 100%    0% / 0% / 0%    2.8 / 4.2 / 4.8</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t xml:space="preserve">    EXPERT   100%    0% / 0% / 0%    3.1 / 4.7 / 5.5</t>
+          <t xml:space="preserve">    EXPERT    99%    0% / 0% / 0%    3.0 / 4.5 / 4.9</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t xml:space="preserve">    STRONG    60%    0% / 9% / 31%    3.5 / 5.6 / 6.7</t>
+          <t xml:space="preserve">    STRONG    63%    0% / 8% / 28%    3.5 / 5.4 / 6.2</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t xml:space="preserve">    AVERAGE    0%    10% / 85% / 4%    4.5 / 7.0 / 7.8</t>
+          <t xml:space="preserve">    AVERAGE    0%    8% / 89% / 2%    4.4 / 6.8 / 7.1</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t xml:space="preserve">    NEWCOMER   0%    69% / 30% / 0%    5.2 / 8.0 / -</t>
+          <t xml:space="preserve">    NEWCOMER   0%    70% / 29% / 0%    5.3 / 6.9 / -</t>
         </is>
       </c>
     </row>
@@ -2674,35 +2674,35 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t xml:space="preserve">    FLAWLESS 100%    0% / 0% / 0%    2.8 / 4.6 / 5.4</t>
+          <t xml:space="preserve">    FLAWLESS 100%    0% / 0% / 0%    2.7 / 4.2 / 4.8</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t xml:space="preserve">    EXPERT    82%    0% / 3% / 14%    3.2 / 5.0 / 5.9</t>
+          <t xml:space="preserve">    EXPERT    84%    0% / 3% / 12%    3.3 / 5.0 / 5.6</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t xml:space="preserve">    STRONG     0%    1% / 68% / 30%    3.8 / 6.1 / 6.8</t>
+          <t xml:space="preserve">    STRONG     0%    2% / 65% / 32%    3.7 / 5.8 / 6.7</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t xml:space="preserve">    AVERAGE    0%    58% / 41% / 0%    4.7 / 6.9 / -</t>
+          <t xml:space="preserve">    AVERAGE    0%    53% / 46% / 0%    4.7 / 6.2 / -</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t xml:space="preserve">    NEWCOMER   0%    98% / 1% / 0%    5.1 / - / -</t>
+          <t xml:space="preserve">    NEWCOMER   0%    98% / 2% / 0%    5.0 / - / -</t>
         </is>
       </c>
     </row>
@@ -2724,14 +2724,14 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t xml:space="preserve">  FANNY MENDELSSOHN AND ???  63% / 0%</t>
+          <t xml:space="preserve">  FANNY MENDELSSOHN AND ???  68% / 0%</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t xml:space="preserve">  THE METRONOME       55% / 0%</t>
+          <t xml:space="preserve">  THE METRONOME       63% / 0%</t>
         </is>
       </c>
     </row>
@@ -2746,35 +2746,35 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t xml:space="preserve">  PAGANINI    57% / 64%</t>
+          <t xml:space="preserve">  PAGANINI    61% / 65%</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t xml:space="preserve">  QUANTZ      59% / 61%</t>
+          <t xml:space="preserve">  QUANTZ      66% / 58%</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t xml:space="preserve">  PFUNDT      63% / 54%</t>
+          <t xml:space="preserve">  PFUNDT      66% / 58%</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t xml:space="preserve">  DUPORT      59% / 60%</t>
+          <t xml:space="preserve">  DUPORT      59% / 70%</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t xml:space="preserve">  PUNTO       60% / 59%</t>
+          <t xml:space="preserve">  PUNTO       62% / 64%</t>
         </is>
       </c>
     </row>
@@ -9601,7 +9601,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D166"/>
+  <dimension ref="A1:D168"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" style="33" min="1" max="1"/>
@@ -10089,7 +10089,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>{ 1.6, 3.6, 5.4 }</t>
+          <t>{ 1.6, 3.8, 5.9 }</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -10111,12 +10111,12 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>{ 1, 1.35, 1.65 }</t>
+          <t>{ 1, 1.38, 1.7 }</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>PATH (Beta1 30 Oct) : was 1.6 / 2.1 / 2.7 and 1 / 1.2 / 1.4. The band grows a step a</t>
+          <t>PATH and SIGNATURE GROWS (Beta1 30 Oct) : was 1.6 / 2.1 / 2.7 and 1 / 1.2 / 1.4. The band</t>
         </is>
       </c>
     </row>
@@ -11475,44 +11475,34 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>Musician Traits in the turn battle</t>
+          <t>SIGNATURE GROWS</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>TurnBreathControl</t>
+          <t>TurnJahrCrescendo</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="D92" t="inlineStr">
-        <is>
-          <t>BREATH CONTROL (QUANTZ) : more BREATH from their ATTACK</t>
+          <t>2</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>Musician Traits in the turn battle</t>
+          <t>SIGNATURE GROWS</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>TurnHandCut</t>
+          <t>TurnJahrScale</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="D93" t="inlineStr">
-        <is>
-          <t>TURN OF THE HAND (PFUNDT) : notes taken off the next attack of an enemy their skill hits</t>
+          <t>1.5</t>
         </is>
       </c>
     </row>
@@ -11524,17 +11514,17 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>TurnHandLeast</t>
+          <t>TurnBreathControl</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>never fewer notes left than this (its point is a long phrase,</t>
+          <t>BREATH CONTROL (QUANTZ) : more BREATH from their ATTACK</t>
         </is>
       </c>
     </row>
@@ -11546,7 +11536,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>TurnScarCrescendo</t>
+          <t>TurnHandCut</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
@@ -11556,7 +11546,7 @@
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>THE SCAR (DUPORT) : CRESCENDO after each enemy attack that hurt them</t>
+          <t>TURN OF THE HAND (PFUNDT) : notes taken off the next attack of an enemy their skill hits</t>
         </is>
       </c>
     </row>
@@ -11568,17 +11558,17 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>TurnHuntingCallScale</t>
+          <t>TurnHandLeast</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>1.3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>THE HUNTING CALL (PUNTO) : the musician who plays right after PUNTO in the bar</t>
+          <t>never fewer notes left than this (its point is a long phrase,</t>
         </is>
       </c>
     </row>
@@ -11590,17 +11580,17 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>TurnLessonWindow</t>
+          <t>TurnScarCrescendo</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>0.05</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>THE LESSON (QUANTZ's skill) : seconds added to the PERFECT window of the friend's next skill, never past GOOD</t>
+          <t>THE SCAR (DUPORT) : CRESCENDO after each enemy attack that hurt them</t>
         </is>
       </c>
     </row>
@@ -11612,17 +11602,17 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>TurnLessonShakes</t>
+          <t>TurnHuntingCallScale</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>1.3</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>a ROLL in it needs this many shakes fewer for PERFECT</t>
+          <t>THE HUNTING CALL (PUNTO) : the musician who plays right after PUNTO in the bar</t>
         </is>
       </c>
     </row>
@@ -11634,17 +11624,17 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>TurnLessonScale</t>
+          <t>TurnLessonWindow</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>1.3</t>
+          <t>0.05</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>and the skill plays this much harder</t>
+          <t>THE LESSON (QUANTZ's skill) : seconds added to the PERFECT window of the friend's next skill, never past GOOD</t>
         </is>
       </c>
     </row>
@@ -11656,17 +11646,17 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>TurnShieldKeep</t>
+          <t>TurnLessonShakes</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>0.5</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>SHIELD (DUPORT's skill) : the share of a hit on the friend that DUPORT takes instead</t>
+          <t>a ROLL in it needs this many shakes fewer for PERFECT</t>
         </is>
       </c>
     </row>
@@ -11678,61 +11668,61 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>TurnChakramRepeat</t>
+          <t>TurnLessonScale</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>0.5</t>
+          <t>1.3</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>CHAKRAM (PUNTO's skill) : an enemy the same throw already hit takes this share</t>
+          <t>and the skill plays this much harder</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>PATH</t>
+          <t>Musician Traits in the turn battle</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>TurnBloodScale</t>
+          <t>TurnShieldKeep</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>1.3</t>
+          <t>0.5</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>THE PACT (PAGANINI) : every skill of theirs plays this much harder</t>
+          <t>SHIELD (DUPORT's skill) : the share of a hit on the friend that DUPORT takes instead</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>PATH</t>
+          <t>Musician Traits in the turn battle</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>TurnPactLife</t>
+          <t>TurnChakramRepeat</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>0.5</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>and costs this much life (never the last of it)</t>
+          <t>CHAKRAM (PUNTO's skill) : an enemy the same throw already hit takes this share</t>
         </is>
       </c>
     </row>
@@ -11744,17 +11734,17 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>TurnLastCutScale</t>
+          <t>TurnBloodScale</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1.3</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>CAPRICE No. 24 (PAGANINI) : the last cut of CAPRICE</t>
+          <t>THE PACT (PAGANINI) : every skill of theirs plays this much harder</t>
         </is>
       </c>
     </row>
@@ -11766,17 +11756,17 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>TurnLessonStrong</t>
+          <t>TurnPactLife</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>1.6</t>
+          <t>4</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>THE METHOD (QUANTZ) : a LESSON plays this much harder (TurnLessonScale without it)</t>
+          <t>and costs this much life (never the last of it)</t>
         </is>
       </c>
     </row>
@@ -11788,17 +11778,17 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>TurnLessonEcho</t>
+          <t>TurnLastCutScale</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>0.5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>EVERY EVENING (QUANTZ) : a friend taught plays their next move again at this</t>
+          <t>CAPRICE No. 24 (PAGANINI) : the last cut of CAPRICE</t>
         </is>
       </c>
     </row>
@@ -11810,17 +11800,17 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>TurnShieldThird</t>
+          <t>TurnLessonStrong</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>0.34</t>
+          <t>1.6</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>STRADIVARIUS (DUPORT) : the share of a blow DUPORT takes for a friend (TurnShieldKeep without it)</t>
+          <t>THE METHOD (QUANTZ) : a LESSON plays this much harder (TurnLessonScale without it)</t>
         </is>
       </c>
     </row>
@@ -11832,17 +11822,17 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>TurnCallStrong</t>
+          <t>TurnLessonEcho</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>1.5</t>
+          <t>0.5</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>TALLY-HO (PUNTO) : THE HUNTING CALL (TurnHuntingCallScale without it)</t>
+          <t>EVERY EVENING (QUANTZ) : a friend taught plays their next move again at this</t>
         </is>
       </c>
     </row>
@@ -11854,17 +11844,17 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>TurnHandOneLeast</t>
+          <t>TurnShieldThird</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0.34</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>ONE TURN (PFUNDT) : TURN OF THE HAND leaves this many notes at least (TurnHandLeast without it)</t>
+          <t>STRADIVARIUS (DUPORT) : the share of a blow DUPORT takes for a friend (TurnShieldKeep without it)</t>
         </is>
       </c>
     </row>
@@ -11876,95 +11866,95 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>TurnHandPaukenCut</t>
+          <t>TurnCallStrong</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1.5</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>DIE PAUKEN (PFUNDT) : TURN OF THE HAND takes this many notes (TurnHandCut without it)</t>
+          <t>TALLY-HO (PUNTO) : THE HUNTING CALL (TurnHuntingCallScale without it)</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>INSPIRED</t>
+          <t>PATH</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>TurnInspiredNeed</t>
+          <t>TurnHandOneLeast</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>ONE TURN (PFUNDT) : TURN OF THE HAND leaves this many notes at least (TurnHandLeast without it)</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>INSPIRED</t>
+          <t>PATH</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>TurnInspiredBreath</t>
+          <t>TurnHandPaukenCut</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
           <t>2</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>DIE PAUKEN (PFUNDT) : TURN OF THE HAND takes this many notes (TurnHandCut without it)</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>The hidden musicians</t>
+          <t>INSPIRED</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>TurnByEarScale</t>
+          <t>TurnInspiredNeed</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>1.5</t>
-        </is>
-      </c>
-      <c r="D113" t="inlineStr">
-        <is>
-          <t>BY EAR (MALI) : against an enemy that is OFF-BEAT</t>
+          <t>4</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>The hidden musicians</t>
+          <t>INSPIRED</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>TurnHeldNoteShare</t>
+          <t>TurnInspiredBreath</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>0.4</t>
-        </is>
-      </c>
-      <c r="D114" t="inlineStr">
-        <is>
-          <t>HELD NOTE (CHAI) : his ATTACK hits again for this share</t>
+          <t>2</t>
         </is>
       </c>
     </row>
@@ -11976,17 +11966,17 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>TurnStepBetterScale</t>
+          <t>TurnByEarScale</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>1.3</t>
+          <t>1.5</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>ONE STEP BETTER (NUAN) : against an enemy whose next attack is long</t>
+          <t>BY EAR (MALI) : against an enemy that is OFF-BEAT</t>
         </is>
       </c>
     </row>
@@ -11998,17 +11988,17 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>TurnLongNotes</t>
+          <t>TurnHeldNoteShare</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>0.4</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>long = this many notes or more (Beta1 29 Oct : was an f note)</t>
+          <t>HELD NOTE (CHAI) : his ATTACK hits again for this share</t>
         </is>
       </c>
     </row>
@@ -12020,29 +12010,29 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>TurnThunderSoften</t>
+          <t>TurnStepBetterScale</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1.3</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>THE WHOLE FLOOR (BORIS) : taken off each note of the enemy's next attack</t>
+          <t>ONE STEP BETTER (NUAN) : against an enemy whose next attack is long</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>ARCHIVE</t>
+          <t>The hidden musicians</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>EchoesPerWin</t>
+          <t>TurnLongNotes</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
@@ -12052,29 +12042,29 @@
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>each fight won</t>
+          <t>long = this many notes or more (Beta1 29 Oct : was an f note)</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>ARCHIVE</t>
+          <t>The hidden musicians</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>EchoesPerFloor</t>
+          <t>TurnThunderSoften</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>each floor cleared</t>
+          <t>THE WHOLE FLOOR (BORIS) : taken off each note of the enemy's next attack</t>
         </is>
       </c>
     </row>
@@ -12086,17 +12076,17 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>EchoesRunWon</t>
+          <t>EchoesPerWin</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>3</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>the whole run won</t>
+          <t>each fight won</t>
         </is>
       </c>
     </row>
@@ -12108,17 +12098,17 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>EchoesMaestro</t>
+          <t>EchoesPerFloor</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>1.5</t>
+          <t>10</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>MAESTRO pays more</t>
+          <t>each floor cleared</t>
         </is>
       </c>
     </row>
@@ -12130,17 +12120,17 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>ArchiveLifePerLevel</t>
+          <t>EchoesRunWon</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>25</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>STRONGER BAND</t>
+          <t>the whole run won</t>
         </is>
       </c>
     </row>
@@ -12152,17 +12142,17 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>ArchiveBreathPerLevel</t>
+          <t>EchoesMaestro</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>1.5</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>DEEP BREATH</t>
+          <t>MAESTRO pays more</t>
         </is>
       </c>
     </row>
@@ -12174,7 +12164,7 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>ArchiveSignaturePerLevel</t>
+          <t>ArchiveLifePerLevel</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
@@ -12184,7 +12174,7 @@
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>WARM UP</t>
+          <t>STRONGER BAND</t>
         </is>
       </c>
     </row>
@@ -12196,17 +12186,17 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>ArchiveShardsPerLevel</t>
+          <t>ArchiveBreathPerLevel</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>SAVINGS</t>
+          <t>DEEP BREATH</t>
         </is>
       </c>
     </row>
@@ -12218,61 +12208,61 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>ArchiveFirstChairTier</t>
+          <t>ArchiveSignaturePerLevel</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>FIRST CHAIR (29 Oct, was FULL STAGE) : the first musician picked starts with their weapon this many tiers up</t>
+          <t>WARM UP</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>Turn Motifs</t>
+          <t>ARCHIVE</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>TurnReedCaseHeal</t>
+          <t>ArchiveShardsPerLevel</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>1.5</t>
+          <t>20</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>REED CASE : wind players' healing</t>
+          <t>SAVINGS</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>Turn Motifs</t>
+          <t>ARCHIVE</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>TurnSpareSticksOffBeat</t>
+          <t>ArchiveFirstChairTier</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>1.5</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>SPARE STICKS : percussion skills' OFF-BEAT</t>
+          <t>FIRST CHAIR (29 Oct, was FULL STAGE) : the first musician picked starts with their weapon this many tiers up</t>
         </is>
       </c>
     </row>
@@ -12284,17 +12274,17 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>TurnPianissimoBreath</t>
+          <t>TurnReedCaseHeal</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>1.5</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>PIANISSIMO : more breath for the first note of an attack parried PERFECT (was a p note)</t>
+          <t>REED CASE : wind players' healing</t>
         </is>
       </c>
     </row>
@@ -12306,17 +12296,17 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>TurnBreathMarkStart</t>
+          <t>TurnSpareSticksOffBeat</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1.5</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>BREATH MARK : more breath at the start of a fight</t>
+          <t>SPARE STICKS : percussion skills' OFF-BEAT</t>
         </is>
       </c>
     </row>
@@ -12328,17 +12318,17 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>TurnTuttiScale</t>
+          <t>TurnPianissimoBreath</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>1.25</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>TUTTI : skills that reach everyone</t>
+          <t>PIANISSIMO : more breath for the first note of an attack parried PERFECT (was a p note)</t>
         </is>
       </c>
     </row>
@@ -12350,17 +12340,17 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>TurnRubatoMiss</t>
+          <t>TurnBreathMarkStart</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>0.6</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>RUBATO : a skill note you MISS still plays at this (step 12)</t>
+          <t>BREATH MARK : more breath at the start of a fight</t>
         </is>
       </c>
     </row>
@@ -12372,17 +12362,17 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>TurnCrescendoStart</t>
+          <t>TurnTuttiScale</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>1.25</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>CRESCENDO : stacks on every musician at the start</t>
+          <t>TUTTI : skills that reach everyone</t>
         </is>
       </c>
     </row>
@@ -12394,17 +12384,17 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>TurnSforzandoScale</t>
+          <t>TurnRubatoMiss</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>1.3</t>
+          <t>0.6</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>SFORZANDO : the PERFECT last note of a skill (was an f note)</t>
+          <t>RUBATO : a skill note you MISS still plays at this (step 12)</t>
         </is>
       </c>
     </row>
@@ -12416,17 +12406,17 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>TurnOvertureScale</t>
+          <t>TurnCrescendoStart</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>OVERTURE : the band's first hit of a fight</t>
+          <t>CRESCENDO : stacks on every musician at the start</t>
         </is>
       </c>
     </row>
@@ -12438,17 +12428,17 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>TurnCounterpointScale</t>
+          <t>TurnSforzandoScale</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1.3</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>COUNTERPOINT : the COUNTER</t>
+          <t>SFORZANDO : the PERFECT last note of a skill (was an f note)</t>
         </is>
       </c>
     </row>
@@ -12460,7 +12450,7 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>TurnAccelerandoShakes</t>
+          <t>TurnOvertureScale</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
@@ -12470,7 +12460,7 @@
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>ACCELERANDO : each shake of a roll counts this many</t>
+          <t>OVERTURE : the band's first hit of a fight</t>
         </is>
       </c>
     </row>
@@ -12482,7 +12472,7 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>TurnGraceTimes</t>
+          <t>TurnCounterpointScale</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
@@ -12492,7 +12482,7 @@
       </c>
       <c r="D138" t="inlineStr">
         <is>
-          <t>GRACE NOTE : a spark that lands does its skill this many times</t>
+          <t>COUNTERPOINT : the COUNTER</t>
         </is>
       </c>
     </row>
@@ -12504,7 +12494,7 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>TurnMarcatoOffBeat</t>
+          <t>TurnAccelerandoShakes</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
@@ -12514,7 +12504,7 @@
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>MARCATO : a PERFECT attack's OFF-BEAT, times this</t>
+          <t>ACCELERANDO : each shake of a roll counts this many</t>
         </is>
       </c>
     </row>
@@ -12526,17 +12516,17 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>TurnConBrioNeed</t>
+          <t>TurnGraceTimes</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D140" t="inlineStr">
         <is>
-          <t>CON BRIO : PERFECTs the SIGNATURE needs instead</t>
+          <t>GRACE NOTE : a spark that lands does its skill this many times</t>
         </is>
       </c>
     </row>
@@ -12548,17 +12538,17 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>TurnCodaBelow</t>
+          <t>TurnMarcatoOffBeat</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>0.25</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>CODA : an enemy under this share of its life</t>
+          <t>MARCATO : a PERFECT attack's OFF-BEAT, times this</t>
         </is>
       </c>
     </row>
@@ -12570,61 +12560,61 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>TurnCodaScale</t>
+          <t>TurnConBrioNeed</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>1.5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="D142" t="inlineStr">
         <is>
-          <t>takes this much more</t>
+          <t>CON BRIO : PERFECTs the SIGNATURE needs instead</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>ONE BAR motifs</t>
+          <t>Turn Motifs</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>TurnDownbeatScale</t>
+          <t>TurnCodaBelow</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>1.5</t>
+          <t>0.25</t>
         </is>
       </c>
       <c r="D143" t="inlineStr">
         <is>
-          <t>DOWNBEAT : the first move of a bar</t>
+          <t>CODA : an enemy under this share of its life</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>ONE BAR motifs</t>
+          <t>Turn Motifs</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>TurnEntranceScale</t>
+          <t>TurnCodaScale</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1.5</t>
         </is>
       </c>
       <c r="D144" t="inlineStr">
         <is>
-          <t>ENTRANCE (29 Oct, CALL is gone) : each musician's first move of a fight. Was : a called musician's first bar</t>
+          <t>takes this much more</t>
         </is>
       </c>
     </row>
@@ -12636,17 +12626,17 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>TurnGreenRoomHeal</t>
+          <t>TurnDownbeatScale</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1.5</t>
         </is>
       </c>
       <c r="D145" t="inlineStr">
         <is>
-          <t>GREEN ROOM (29 Oct, the BENCH is gone) : life back for the most hurt musician standing at the end of a</t>
+          <t>DOWNBEAT : the first move of a bar</t>
         </is>
       </c>
     </row>
@@ -12658,7 +12648,7 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>TurnUnisonScale</t>
+          <t>TurnEntranceScale</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
@@ -12668,51 +12658,51 @@
       </c>
       <c r="D146" t="inlineStr">
         <is>
-          <t>UNISON : the last ATTACK of a bar that all goes at one enemy</t>
+          <t>ENTRANCE (29 Oct, CALL is gone) : each musician's first move of a fight. Was : a called musician's first bar</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>Turn Feel</t>
+          <t>ONE BAR motifs</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>TurnRingTime</t>
+          <t>TurnGreenRoomHeal</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>1.1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="D147" t="inlineStr">
         <is>
-          <t>from a note showing to the moment to swipe</t>
+          <t>GREEN ROOM (29 Oct, the BENCH is gone) : life back for the most hurt musician standing at the end of a</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>Turn Feel</t>
+          <t>ONE BAR motifs</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>TurnLateReveal</t>
+          <t>TurnUnisonScale</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>0.5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D148" t="inlineStr">
         <is>
-          <t>FALSE NOTES (STATIC) : its hidden note shows its arrow once the ring is this far closed</t>
+          <t>UNISON : the last ATTACK of a bar that all goes at one enemy</t>
         </is>
       </c>
     </row>
@@ -12724,17 +12714,17 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>MaestroTurnRingTime</t>
+          <t>TurnRingTime</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>0.8</t>
+          <t>1.1</t>
         </is>
       </c>
       <c r="D149" t="inlineStr">
         <is>
-          <t>MAESTRO</t>
+          <t>from a note showing to the moment to swipe</t>
         </is>
       </c>
     </row>
@@ -12746,17 +12736,17 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>TurnNoteGap</t>
+          <t>TurnLateReveal</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>0.55</t>
+          <t>0.5</t>
         </is>
       </c>
       <c r="D150" t="inlineStr">
         <is>
-          <t>between the notes of one enemy attack</t>
+          <t>FALSE NOTES (STATIC) : its hidden note shows its arrow once the ring is this far closed</t>
         </is>
       </c>
     </row>
@@ -12768,7 +12758,7 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>TurnPause</t>
+          <t>MaestroTurnRingTime</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
@@ -12778,7 +12768,7 @@
       </c>
       <c r="D151" t="inlineStr">
         <is>
-          <t>after a turn, before the next one starts</t>
+          <t>MAESTRO</t>
         </is>
       </c>
     </row>
@@ -12790,17 +12780,17 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>TurnHitStop</t>
+          <t>TurnNoteGap</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>0.075</t>
+          <t>0.55</t>
         </is>
       </c>
       <c r="D152" t="inlineStr">
         <is>
-          <t>the band and TACET freeze for a moment on a PERFECT</t>
+          <t>between the notes of one enemy attack</t>
         </is>
       </c>
     </row>
@@ -12812,17 +12802,17 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>TurnStrikeTime</t>
+          <t>TurnPause</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>0.62</t>
+          <t>0.8</t>
         </is>
       </c>
       <c r="D153" t="inlineStr">
         <is>
-          <t>ONE BAR : how long an ATTACK's lunge takes, there and back (Beta1 : slower, smoother)</t>
+          <t>after a turn, before the next one starts</t>
         </is>
       </c>
     </row>
@@ -12834,17 +12824,17 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>TurnStrikeImpact</t>
+          <t>TurnHitStop</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>0.24</t>
+          <t>0.075</t>
         </is>
       </c>
       <c r="D154" t="inlineStr">
         <is>
-          <t>when in it the hit lands</t>
+          <t>the band and TACET freeze for a moment on a PERFECT</t>
         </is>
       </c>
     </row>
@@ -12856,17 +12846,17 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>TurnStrikeStop</t>
+          <t>TurnStrikeTime</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>0.08</t>
+          <t>0.62</t>
         </is>
       </c>
       <c r="D155" t="inlineStr">
         <is>
-          <t>the freeze when it lands</t>
+          <t>ONE BAR : how long an ATTACK's lunge takes, there and back (Beta1 : slower, smoother)</t>
         </is>
       </c>
     </row>
@@ -12878,17 +12868,17 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>TurnNumberTime</t>
+          <t>TurnStrikeImpact</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>0.24</t>
         </is>
       </c>
       <c r="D156" t="inlineStr">
         <is>
-          <t>a damage number stays this long (Beta1 round 4, pixel numbers)</t>
+          <t>when in it the hit lands</t>
         </is>
       </c>
     </row>
@@ -12900,17 +12890,17 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>TurnBigHit</t>
+          <t>TurnStrikeStop</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>0.08</t>
         </is>
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t>from this much damage it is drawn bigger</t>
+          <t>the freeze when it lands</t>
         </is>
       </c>
     </row>
@@ -12922,17 +12912,17 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>TurnNumberCell</t>
+          <t>TurnNumberTime</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>4.5</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t>one cell of a digit (5 x 7 cells) in pixels (round 4 : 25% smaller, was 6)</t>
+          <t>a damage number stays this long (Beta1 round 4, pixel numbers)</t>
         </is>
       </c>
     </row>
@@ -12944,17 +12934,17 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>TurnNumberBigCell</t>
+          <t>TurnBigHit</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>18</t>
         </is>
       </c>
       <c r="D159" t="inlineStr">
         <is>
-          <t>the same for a big hit (was 8)</t>
+          <t>from this much damage it is drawn bigger</t>
         </is>
       </c>
     </row>
@@ -12966,17 +12956,17 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>TurnDissolveTime</t>
+          <t>TurnNumberCell</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>4.5</t>
         </is>
       </c>
       <c r="D160" t="inlineStr">
         <is>
-          <t>an enemy SILENCED dissolves into TACET's hole in this long</t>
+          <t>one cell of a digit (5 x 7 cells) in pixels (round 4 : 25% smaller, was 6)</t>
         </is>
       </c>
     </row>
@@ -12988,17 +12978,17 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>TurnCutInTime</t>
+          <t>TurnNumberBigCell</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>1.3</t>
+          <t>6</t>
         </is>
       </c>
       <c r="D161" t="inlineStr">
         <is>
-          <t>the SIGNATURE's CUT-IN, before its strokes (Beta1 round 4, the old duel's picture)</t>
+          <t>the same for a big hit (was 8)</t>
         </is>
       </c>
     </row>
@@ -13010,17 +13000,17 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>TurnKillStop</t>
+          <t>TurnDissolveTime</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>0.18</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="D162" t="inlineStr">
         <is>
-          <t>the freeze when an enemy falls silent</t>
+          <t>an enemy SILENCED dissolves into TACET's hole in this long</t>
         </is>
       </c>
     </row>
@@ -13032,17 +13022,17 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>TurnEndTime</t>
+          <t>TurnCutInTime</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>2.2</t>
+          <t>1.3</t>
         </is>
       </c>
       <c r="D163" t="inlineStr">
         <is>
-          <t>the win or lose banner stays this long</t>
+          <t>the SIGNATURE's CUT-IN, before its strokes (Beta1 round 4, the old duel's picture)</t>
         </is>
       </c>
     </row>
@@ -13054,17 +13044,17 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>TurnSparkGap</t>
+          <t>TurnKillStop</t>
         </is>
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>0.3</t>
+          <t>0.18</t>
         </is>
       </c>
       <c r="D164" t="inlineStr">
         <is>
-          <t>a spark comes this soon after the note before it</t>
+          <t>the freeze when an enemy falls silent</t>
         </is>
       </c>
     </row>
@@ -13076,17 +13066,17 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>TurnHoldTime</t>
+          <t>TurnEndTime</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>0.8</t>
+          <t>2.2</t>
         </is>
       </c>
       <c r="D165" t="inlineStr">
         <is>
-          <t>how long a HOLD note wants holding (the button kept down, the baton may move : Beta1 29 Oct)</t>
+          <t>the win or lose banner stays this long</t>
         </is>
       </c>
     </row>
@@ -13098,15 +13088,59 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
+          <t>TurnSparkGap</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>0.3</t>
+        </is>
+      </c>
+      <c r="D166" t="inlineStr">
+        <is>
+          <t>a spark comes this soon after the note before it</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>Turn Feel</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>TurnHoldTime</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>0.8</t>
+        </is>
+      </c>
+      <c r="D167" t="inlineStr">
+        <is>
+          <t>how long a HOLD note wants holding (the button kept down, the baton may move : Beta1 29 Oct)</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>Turn Feel</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
           <t>TurnRollTime</t>
         </is>
       </c>
-      <c r="C166" t="inlineStr">
+      <c r="C168" t="inlineStr">
         <is>
           <t>1.2</t>
         </is>
       </c>
-      <c r="D166" t="inlineStr">
+      <c r="D168" t="inlineStr">
         <is>
           <t>how long a ROLL note lasts</t>
         </is>

</xml_diff>

<commit_message>
Beta1 : block 2 part 8, BONDS from the legends' real history (block 2 done)
Five ties (Data/Bond.cs), checked : Beethoven with DUPORT (the cello sonatas
Op. 5, Berlin 1796) and PUNTO (the Horn Sonata Op. 17, Vienna 1800), Bach with
QUANTZ (the king's theme of the Musical Offering), Fanny with PFUNDT (Felix's
Gewandhaus, 1835), and PAGANINI against THE DEVIL'S STRING. A tied legend's
first move of every fight is x1.5 (PAGANINI hits the devil x1.5). The audition
shows the tie over the column and says it when picked, a fight opens with the
legend's line. A SIGNATURE made cheaper by the ties was the first try, it made
runs far too easy with STORM. TACET's floors 2 and 3 grew a little more : over
24 seeds the run is as hard as before block 2 (63.1 percent, 63.8 before,
MAESTRO EXPERT 82.6 and 82.0). turncheck 138/138, savecheck 33/33.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LkyThr8Ag8ofurL2payU71
</commit_message>
<xml_diff>
--- a/docs/TACET_Balance.xlsx
+++ b/docs/TACET_Balance.xlsx
@@ -2335,112 +2335,112 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t xml:space="preserve">  FLAWLESS  FLOOR 1  EARLY 100%  2.0b   0%   LATE  100%  2.2b   6%   ELITE 100%  3.0b   8%   BOSS  100%  5.4b  13%   </t>
+          <t xml:space="preserve">  FLAWLESS  FLOOR 1  EARLY 100%  2.0b   0%   LATE  100%  2.2b   6%   ELITE 100%  3.0b   8%   BOSS  100%  5.3b  13%   </t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t xml:space="preserve">  FLAWLESS  FLOOR 2  EARLY 100%  3.0b   8%   LATE  100%  4.5b  11%   ELITE 100%  5.5b  15%   BOSS  100%  9.9b  17%   </t>
+          <t xml:space="preserve">  FLAWLESS  FLOOR 2  EARLY 100%  3.0b   8%   LATE  100%  4.7b  11%   ELITE 100%  5.4b  15%   BOSS  100%  9.7b  16%   </t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t xml:space="preserve">  FLAWLESS  FLOOR 3  EARLY 100%  4.1b  11%   LATE  100%  5.0b  14%   ELITE 100%  6.0b  16%   BOSS  100% 10.7b  16%   </t>
+          <t xml:space="preserve">  FLAWLESS  FLOOR 3  EARLY 100%  4.2b  11%   LATE  100%  5.0b  14%   ELITE 100%  6.0b  16%   BOSS  100% 10.5b  16%   </t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t xml:space="preserve">  EXPERT    FLOOR 1  EARLY 100%  1.1b   3%   LATE  100%  2.0b   7%   ELITE 100%  2.0b   7%   BOSS  100%  3.7b  11%   </t>
+          <t xml:space="preserve">  EXPERT    FLOOR 1  EARLY 100%  1.1b   3%   LATE  100%  2.0b   7%   ELITE 100%  2.0b   7%   BOSS  100%  3.7b  10%   </t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t xml:space="preserve">  EXPERT    FLOOR 2  EARLY 100%  3.2b  12%   LATE  100%  4.1b  16%   ELITE 100%  4.6b  17%   BOSS  100%  8.0b  22%   </t>
+          <t xml:space="preserve">  EXPERT    FLOOR 2  EARLY 100%  3.1b  12%   LATE  100%  4.1b  16%   ELITE 100%  4.6b  16%   BOSS  100%  7.7b  23%   </t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t xml:space="preserve">  EXPERT    FLOOR 3  EARLY 100%  4.7b  18%   LATE  100%  5.6b  22%   ELITE 100%  7.0b  23%   BOSS   99% 12.7b  25%   </t>
+          <t xml:space="preserve">  EXPERT    FLOOR 3  EARLY 100%  4.7b  18%   LATE  100%  5.8b  21%   ELITE 100%  7.0b  22%   BOSS  100% 12.4b  24%   </t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t xml:space="preserve">  STRONG    FLOOR 1  EARLY 100%  1.3b   5%   LATE  100%  2.2b  10%   ELITE 100%  2.4b  11%   BOSS  100%  4.1b  17%   </t>
+          <t xml:space="preserve">  STRONG    FLOOR 1  EARLY 100%  1.3b   4%   LATE  100%  2.2b  10%   ELITE 100%  2.4b  11%   BOSS  100%  4.0b  17%   </t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t xml:space="preserve">  STRONG    FLOOR 2  EARLY 100%  3.5b  18%   LATE  100%  4.6b  22%   ELITE  99%  5.7b  23%   BOSS   96% 10.8b  38%   </t>
+          <t xml:space="preserve">  STRONG    FLOOR 2  EARLY 100%  3.6b  18%   LATE  100%  4.8b  23%   ELITE 100%  5.8b  24%   BOSS   96%  9.9b  34%   </t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t xml:space="preserve">  STRONG    FLOOR 3  EARLY 100%  5.9b  26%   LATE  100%  7.4b  27%   ELITE  95% 10.0b  37%   BOSS   73% 15.4b  54%   </t>
+          <t xml:space="preserve">  STRONG    FLOOR 3  EARLY 100%  5.9b  26%   LATE  100%  7.4b  26%   ELITE  97% 10.0b  33%   BOSS   70% 16.0b  57%   </t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t xml:space="preserve">  AVERAGE   FLOOR 1  EARLY 100%  1.8b   9%   LATE  100%  2.9b  18%   ELITE 100%  3.1b  20%   BOSS   98%  5.4b  34%   </t>
+          <t xml:space="preserve">  AVERAGE   FLOOR 1  EARLY 100%  1.7b   9%   LATE  100%  2.9b  18%   ELITE 100%  3.2b  20%   BOSS   99%  5.3b  32%   </t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t xml:space="preserve">  AVERAGE   FLOOR 2  EARLY  99%  5.3b  31%   LATE   96%  7.9b  41%   ELITE  77% 10.6b  58%   BOSS   22% 11.3b  89%   </t>
+          <t xml:space="preserve">  AVERAGE   FLOOR 2  EARLY 100%  5.3b  32%   LATE   95%  7.5b  43%   ELITE  77% 10.2b  57%   BOSS   24% 11.4b  90%   </t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t xml:space="preserve">  AVERAGE   FLOOR 3  EARLY  67%  9.5b  64%   LATE   38%  8.6b  84%   ELITE  13%  9.9b  94%   BOSS    0%  6.5b 100%   </t>
+          <t xml:space="preserve">  AVERAGE   FLOOR 3  EARLY  62%  9.7b  69%   LATE   36%  9.4b  84%   ELITE  13% 10.0b  95%   BOSS    0%  6.9b 100%   </t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t xml:space="preserve">  NEWCOMER  FLOOR 1  EARLY 100%  2.1b  14%   LATE  100%  3.8b  29%   ELITE 100%  4.1b  30%   BOSS   65%  8.1b  72%   </t>
+          <t xml:space="preserve">  NEWCOMER  FLOOR 1  EARLY 100%  2.1b  14%   LATE  100%  3.8b  30%   ELITE 100%  4.2b  31%   BOSS   77%  7.7b  68%   </t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t xml:space="preserve">  NEWCOMER  FLOOR 2  EARLY  81%  8.5b  61%   LATE   29%  8.3b  89%   ELITE   5%  9.1b  98%   BOSS    0%  6.3b  99%   </t>
+          <t xml:space="preserve">  NEWCOMER  FLOOR 2  EARLY  84%  8.4b  59%   LATE   33%  8.6b  88%   ELITE  10%  9.7b  96%   BOSS    0%  6.5b  99%   </t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t xml:space="preserve">  NEWCOMER  FLOOR 3  EARLY   1%  5.5b  99%   LATE    0%  3.7b 100%   ELITE   0%  4.5b 100%   BOSS    0%  3.4b 100%   </t>
+          <t xml:space="preserve">  NEWCOMER  FLOOR 3  EARLY   3%  5.6b  99%   LATE    0%  4.0b 100%   ELITE   0%  4.6b 100%   BOSS    0%  3.5b 100%   </t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t xml:space="preserve">  DAMAGE SHARE in all of the fights above : ATTACK 13%  SKILLS 86%</t>
+          <t xml:space="preserve">  DAMAGE SHARE in all of the fights above : ATTACK 12%  SKILLS 87%</t>
         </is>
       </c>
     </row>
@@ -2462,28 +2462,28 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t xml:space="preserve">  EXPERT    31 /  66 /   1 /   0   x1.65</t>
+          <t xml:space="preserve">  EXPERT    33 /  64 /   1 /   0   x1.66</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t xml:space="preserve">  STRONG     3 /  49 /  44 /   2   x1.39</t>
+          <t xml:space="preserve">  STRONG     3 /  49 /  44 /   2   x1.40</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t xml:space="preserve">  AVERAGE    0 /   4 /  63 /  31   x1.18</t>
+          <t xml:space="preserve">  AVERAGE    0 /   5 /  62 /  32   x1.18</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t xml:space="preserve">  NEWCOMER   0 /   0 /  35 /  63   x1.09</t>
+          <t xml:space="preserve">  NEWCOMER   0 /   0 /  34 /  64   x1.09</t>
         </is>
       </c>
     </row>
@@ -2498,119 +2498,119 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t xml:space="preserve">  HUSH                   98%  7.1b    100%  4.8b    </t>
+          <t xml:space="preserve">  HUSH                   94%  7.7b    100%  4.8b    </t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t xml:space="preserve">  DEAD AIR               96%  7.2b    100%  4.7b    </t>
+          <t xml:space="preserve">  DEAD AIR               92%  7.6b    100%  4.8b    </t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t xml:space="preserve">  THE LULL               97%  7.8b    100%  4.9b    </t>
+          <t xml:space="preserve">  THE LULL               97%  7.8b    100%  5.0b    </t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t xml:space="preserve">  STATIC                 92%  7.3b    100%  4.6b    </t>
+          <t xml:space="preserve">  STATIC                 94%  7.5b    100%  4.7b    </t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t xml:space="preserve">  THE MUTE CHOIR         93%  10.1b    100%  5.9b    </t>
+          <t xml:space="preserve">  THE MUTE CHOIR         92%  10.6b    100%  6.0b    </t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t xml:space="preserve">  WHITE NOISE            66%  8.5b    100%  5.4b    </t>
+          <t xml:space="preserve">  WHITE NOISE            64%  9.0b     99%  5.5b    </t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t xml:space="preserve">  REQUIEM                 0%  7.1b     67%  16.1b    </t>
+          <t xml:space="preserve">  REQUIEM                 0%  6.3b     63%  15.9b    </t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t xml:space="preserve">  THE NAMELESS MASTER     3%  10.6b     94%  14.6b    </t>
+          <t xml:space="preserve">  THE NAMELESS MASTER     5%  11.0b     94%  14.8b    </t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t xml:space="preserve">  THE DEVIL'S STRING      0%  5.6b     43%  15.2b    </t>
+          <t xml:space="preserve">  THE DEVIL'S STRING      0%  5.6b     57%  13.5b    </t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t xml:space="preserve">  ROOM TONE              97%  7.5b    100%  4.9b    </t>
+          <t xml:space="preserve">  ROOM TONE              95%  7.2b    100%  5.0b    </t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  THE CUE                96%  7.8b    100%  4.9b    </t>
+          <t xml:space="preserve">  THE CUE                95%  8.1b    100%  5.0b    </t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t xml:space="preserve">  THE DAMPER             94%  7.7b    100%  4.8b    </t>
+          <t xml:space="preserve">  THE DAMPER             93%  7.8b    100%  4.8b    </t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t xml:space="preserve">  STUTTER                99%  7.0b    100%  4.4b    </t>
+          <t xml:space="preserve">  STUTTER                98%  6.9b    100%  4.5b    </t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t xml:space="preserve">  THE ROUND              76%  12.4b    100%  6.0b    </t>
+          <t xml:space="preserve">  THE ROUND              80%  12.1b    100%  5.9b    </t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t xml:space="preserve">  THE DEAF CROWN          0%  5.8b     61%  19.6b    </t>
+          <t xml:space="preserve">  THE DEAF CROWN          0%  5.8b     46%  18.6b    </t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t xml:space="preserve">  THE STAFF               0%  7.0b     73%  17.3b    </t>
+          <t xml:space="preserve">  THE STAFF               0%  7.0b     63%  16.9b    </t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t xml:space="preserve">  THE BLIND CANTOR        0%  6.7b     77%  15.4b    </t>
+          <t xml:space="preserve">  THE BLIND CANTOR        0%  6.2b     61%  15.7b    </t>
         </is>
       </c>
     </row>
@@ -2632,35 +2632,35 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t xml:space="preserve">    FLAWLESS 100%    0% / 0% / 0%    2.8 / 4.2 / 4.8</t>
+          <t xml:space="preserve">    FLAWLESS 100%    0% / 0% / 0%    2.7 / 4.1 / 4.7</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t xml:space="preserve">    EXPERT    99%    0% / 0% / 0%    3.0 / 4.5 / 4.9</t>
+          <t xml:space="preserve">    EXPERT   100%    0% / 0% / 0%    3.0 / 4.5 / 5.0</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t xml:space="preserve">    STRONG    63%    0% / 8% / 28%    3.5 / 5.4 / 6.2</t>
+          <t xml:space="preserve">    STRONG    66%    0% / 7% / 26%    3.3 / 5.3 / 6.1</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t xml:space="preserve">    AVERAGE    0%    8% / 89% / 2%    4.4 / 6.8 / 7.1</t>
+          <t xml:space="preserve">    AVERAGE    0%    8% / 88% / 3%    4.3 / 6.7 / 7.3</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t xml:space="preserve">    NEWCOMER   0%    70% / 29% / 0%    5.3 / 6.9 / -</t>
+          <t xml:space="preserve">    NEWCOMER   0%    69% / 30% / 0%    5.1 / 7.1 / -</t>
         </is>
       </c>
     </row>
@@ -2674,35 +2674,35 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t xml:space="preserve">    FLAWLESS 100%    0% / 0% / 0%    2.7 / 4.2 / 4.8</t>
+          <t xml:space="preserve">    FLAWLESS 100%    0% / 0% / 0%    2.7 / 4.3 / 4.8</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t xml:space="preserve">    EXPERT    84%    0% / 3% / 12%    3.3 / 5.0 / 5.6</t>
+          <t xml:space="preserve">    EXPERT    79%    0% / 4% / 16%    3.1 / 4.9 / 5.5</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t xml:space="preserve">    STRONG     0%    2% / 65% / 32%    3.7 / 5.8 / 6.7</t>
+          <t xml:space="preserve">    STRONG     0%    0% / 65% / 34%    3.6 / 5.8 / 6.4</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t xml:space="preserve">    AVERAGE    0%    53% / 46% / 0%    4.7 / 6.2 / -</t>
+          <t xml:space="preserve">    AVERAGE    0%    58% / 41% / 0%    4.5 / 6.3 / -</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t xml:space="preserve">    NEWCOMER   0%    98% / 2% / 0%    5.0 / - / -</t>
+          <t xml:space="preserve">    NEWCOMER   0%    98% / 1% / 0%    4.9 / - / -</t>
         </is>
       </c>
     </row>
@@ -2717,21 +2717,21 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t xml:space="preserve">  THE UNHEARING       60% / 0%</t>
+          <t xml:space="preserve">  THE UNHEARING       67% / 0%</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t xml:space="preserve">  FANNY MENDELSSOHN AND ???  68% / 0%</t>
+          <t xml:space="preserve">  FANNY MENDELSSOHN AND ???  64% / 0%</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t xml:space="preserve">  THE METRONOME       63% / 0%</t>
+          <t xml:space="preserve">  THE METRONOME       59% / 0%</t>
         </is>
       </c>
     </row>
@@ -2746,35 +2746,35 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t xml:space="preserve">  PAGANINI    61% / 65%</t>
+          <t xml:space="preserve">  PAGANINI    65% / 67%</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t xml:space="preserve">  QUANTZ      66% / 58%</t>
+          <t xml:space="preserve">  QUANTZ      68% / 63%</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t xml:space="preserve">  PFUNDT      66% / 58%</t>
+          <t xml:space="preserve">  PFUNDT      64% / 68%</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t xml:space="preserve">  DUPORT      59% / 70%</t>
+          <t xml:space="preserve">  DUPORT      65% / 68%</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t xml:space="preserve">  PUNTO       62% / 64%</t>
+          <t xml:space="preserve">  PUNTO       67% / 64%</t>
         </is>
       </c>
     </row>
@@ -9601,7 +9601,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D168"/>
+  <dimension ref="A1:D170"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" style="33" min="1" max="1"/>
@@ -10089,7 +10089,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>{ 1.6, 3.8, 5.9 }</t>
+          <t>{ 1.6, 3.85, 6 }</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -10111,12 +10111,12 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>{ 1, 1.38, 1.7 }</t>
+          <t>{ 1, 1.39, 1.72 }</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>PATH and SIGNATURE GROWS (Beta1 30 Oct) : was 1.6 / 2.1 / 2.7 and 1 / 1.2 / 1.4. The band</t>
+          <t>PATH, SIGNATURE GROWS and BONDS (Beta1 30 Oct) : was 1.6 / 2.1 / 2.7 and 1 / 1.2 / 1.4. The</t>
         </is>
       </c>
     </row>
@@ -11509,44 +11509,39 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>Musician Traits in the turn battle</t>
+          <t>BONDS</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>TurnBreathControl</t>
+          <t>TurnBondScale</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="D94" t="inlineStr">
-        <is>
-          <t>BREATH CONTROL (QUANTZ) : more BREATH from their ATTACK</t>
+          <t>1.5</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>Musician Traits in the turn battle</t>
+          <t>BONDS</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>TurnHandCut</t>
+          <t>TurnBondLineTime</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>TURN OF THE HAND (PFUNDT) : notes taken off the next attack of an enemy their skill hits</t>
+          <t>seconds a tied legend's line shows as the fight starts</t>
         </is>
       </c>
     </row>
@@ -11558,17 +11553,17 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>TurnHandLeast</t>
+          <t>TurnBreathControl</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>never fewer notes left than this (its point is a long phrase,</t>
+          <t>BREATH CONTROL (QUANTZ) : more BREATH from their ATTACK</t>
         </is>
       </c>
     </row>
@@ -11580,7 +11575,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>TurnScarCrescendo</t>
+          <t>TurnHandCut</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
@@ -11590,7 +11585,7 @@
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>THE SCAR (DUPORT) : CRESCENDO after each enemy attack that hurt them</t>
+          <t>TURN OF THE HAND (PFUNDT) : notes taken off the next attack of an enemy their skill hits</t>
         </is>
       </c>
     </row>
@@ -11602,17 +11597,17 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>TurnHuntingCallScale</t>
+          <t>TurnHandLeast</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>1.3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>THE HUNTING CALL (PUNTO) : the musician who plays right after PUNTO in the bar</t>
+          <t>never fewer notes left than this (its point is a long phrase,</t>
         </is>
       </c>
     </row>
@@ -11624,17 +11619,17 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>TurnLessonWindow</t>
+          <t>TurnScarCrescendo</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>0.05</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>THE LESSON (QUANTZ's skill) : seconds added to the PERFECT window of the friend's next skill, never past GOOD</t>
+          <t>THE SCAR (DUPORT) : CRESCENDO after each enemy attack that hurt them</t>
         </is>
       </c>
     </row>
@@ -11646,17 +11641,17 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>TurnLessonShakes</t>
+          <t>TurnHuntingCallScale</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>1.3</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>a ROLL in it needs this many shakes fewer for PERFECT</t>
+          <t>THE HUNTING CALL (PUNTO) : the musician who plays right after PUNTO in the bar</t>
         </is>
       </c>
     </row>
@@ -11668,17 +11663,17 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>TurnLessonScale</t>
+          <t>TurnLessonWindow</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>1.3</t>
+          <t>0.05</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>and the skill plays this much harder</t>
+          <t>THE LESSON (QUANTZ's skill) : seconds added to the PERFECT window of the friend's next skill, never past GOOD</t>
         </is>
       </c>
     </row>
@@ -11690,17 +11685,17 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>TurnShieldKeep</t>
+          <t>TurnLessonShakes</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>0.5</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>SHIELD (DUPORT's skill) : the share of a hit on the friend that DUPORT takes instead</t>
+          <t>a ROLL in it needs this many shakes fewer for PERFECT</t>
         </is>
       </c>
     </row>
@@ -11712,61 +11707,61 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>TurnChakramRepeat</t>
+          <t>TurnLessonScale</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>0.5</t>
+          <t>1.3</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>CHAKRAM (PUNTO's skill) : an enemy the same throw already hit takes this share</t>
+          <t>and the skill plays this much harder</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>PATH</t>
+          <t>Musician Traits in the turn battle</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>TurnBloodScale</t>
+          <t>TurnShieldKeep</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>1.3</t>
+          <t>0.5</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>THE PACT (PAGANINI) : every skill of theirs plays this much harder</t>
+          <t>SHIELD (DUPORT's skill) : the share of a hit on the friend that DUPORT takes instead</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>PATH</t>
+          <t>Musician Traits in the turn battle</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>TurnPactLife</t>
+          <t>TurnChakramRepeat</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>0.5</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>and costs this much life (never the last of it)</t>
+          <t>CHAKRAM (PUNTO's skill) : an enemy the same throw already hit takes this share</t>
         </is>
       </c>
     </row>
@@ -11778,17 +11773,17 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>TurnLastCutScale</t>
+          <t>TurnBloodScale</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1.3</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>CAPRICE No. 24 (PAGANINI) : the last cut of CAPRICE</t>
+          <t>THE PACT (PAGANINI) : every skill of theirs plays this much harder</t>
         </is>
       </c>
     </row>
@@ -11800,17 +11795,17 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>TurnLessonStrong</t>
+          <t>TurnPactLife</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>1.6</t>
+          <t>4</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>THE METHOD (QUANTZ) : a LESSON plays this much harder (TurnLessonScale without it)</t>
+          <t>and costs this much life (never the last of it)</t>
         </is>
       </c>
     </row>
@@ -11822,17 +11817,17 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>TurnLessonEcho</t>
+          <t>TurnLastCutScale</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>0.5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>EVERY EVENING (QUANTZ) : a friend taught plays their next move again at this</t>
+          <t>CAPRICE No. 24 (PAGANINI) : the last cut of CAPRICE</t>
         </is>
       </c>
     </row>
@@ -11844,17 +11839,17 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>TurnShieldThird</t>
+          <t>TurnLessonStrong</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>0.34</t>
+          <t>1.6</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>STRADIVARIUS (DUPORT) : the share of a blow DUPORT takes for a friend (TurnShieldKeep without it)</t>
+          <t>THE METHOD (QUANTZ) : a LESSON plays this much harder (TurnLessonScale without it)</t>
         </is>
       </c>
     </row>
@@ -11866,17 +11861,17 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>TurnCallStrong</t>
+          <t>TurnLessonEcho</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>1.5</t>
+          <t>0.5</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>TALLY-HO (PUNTO) : THE HUNTING CALL (TurnHuntingCallScale without it)</t>
+          <t>EVERY EVENING (QUANTZ) : a friend taught plays their next move again at this</t>
         </is>
       </c>
     </row>
@@ -11888,17 +11883,17 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>TurnHandOneLeast</t>
+          <t>TurnShieldThird</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0.34</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>ONE TURN (PFUNDT) : TURN OF THE HAND leaves this many notes at least (TurnHandLeast without it)</t>
+          <t>STRADIVARIUS (DUPORT) : the share of a blow DUPORT takes for a friend (TurnShieldKeep without it)</t>
         </is>
       </c>
     </row>
@@ -11910,95 +11905,95 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>TurnHandPaukenCut</t>
+          <t>TurnCallStrong</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1.5</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>DIE PAUKEN (PFUNDT) : TURN OF THE HAND takes this many notes (TurnHandCut without it)</t>
+          <t>TALLY-HO (PUNTO) : THE HUNTING CALL (TurnHuntingCallScale without it)</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>INSPIRED</t>
+          <t>PATH</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>TurnInspiredNeed</t>
+          <t>TurnHandOneLeast</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>ONE TURN (PFUNDT) : TURN OF THE HAND leaves this many notes at least (TurnHandLeast without it)</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>INSPIRED</t>
+          <t>PATH</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>TurnInspiredBreath</t>
+          <t>TurnHandPaukenCut</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
           <t>2</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>DIE PAUKEN (PFUNDT) : TURN OF THE HAND takes this many notes (TurnHandCut without it)</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>The hidden musicians</t>
+          <t>INSPIRED</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>TurnByEarScale</t>
+          <t>TurnInspiredNeed</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>1.5</t>
-        </is>
-      </c>
-      <c r="D115" t="inlineStr">
-        <is>
-          <t>BY EAR (MALI) : against an enemy that is OFF-BEAT</t>
+          <t>4</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>The hidden musicians</t>
+          <t>INSPIRED</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>TurnHeldNoteShare</t>
+          <t>TurnInspiredBreath</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>0.4</t>
-        </is>
-      </c>
-      <c r="D116" t="inlineStr">
-        <is>
-          <t>HELD NOTE (CHAI) : his ATTACK hits again for this share</t>
+          <t>2</t>
         </is>
       </c>
     </row>
@@ -12010,17 +12005,17 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>TurnStepBetterScale</t>
+          <t>TurnByEarScale</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>1.3</t>
+          <t>1.5</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>ONE STEP BETTER (NUAN) : against an enemy whose next attack is long</t>
+          <t>BY EAR (MALI) : against an enemy that is OFF-BEAT</t>
         </is>
       </c>
     </row>
@@ -12032,17 +12027,17 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>TurnLongNotes</t>
+          <t>TurnHeldNoteShare</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>0.4</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>long = this many notes or more (Beta1 29 Oct : was an f note)</t>
+          <t>HELD NOTE (CHAI) : his ATTACK hits again for this share</t>
         </is>
       </c>
     </row>
@@ -12054,29 +12049,29 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>TurnThunderSoften</t>
+          <t>TurnStepBetterScale</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1.3</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>THE WHOLE FLOOR (BORIS) : taken off each note of the enemy's next attack</t>
+          <t>ONE STEP BETTER (NUAN) : against an enemy whose next attack is long</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>ARCHIVE</t>
+          <t>The hidden musicians</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>EchoesPerWin</t>
+          <t>TurnLongNotes</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
@@ -12086,29 +12081,29 @@
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>each fight won</t>
+          <t>long = this many notes or more (Beta1 29 Oct : was an f note)</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>ARCHIVE</t>
+          <t>The hidden musicians</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>EchoesPerFloor</t>
+          <t>TurnThunderSoften</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>each floor cleared</t>
+          <t>THE WHOLE FLOOR (BORIS) : taken off each note of the enemy's next attack</t>
         </is>
       </c>
     </row>
@@ -12120,17 +12115,17 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>EchoesRunWon</t>
+          <t>EchoesPerWin</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>3</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>the whole run won</t>
+          <t>each fight won</t>
         </is>
       </c>
     </row>
@@ -12142,17 +12137,17 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>EchoesMaestro</t>
+          <t>EchoesPerFloor</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>1.5</t>
+          <t>10</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>MAESTRO pays more</t>
+          <t>each floor cleared</t>
         </is>
       </c>
     </row>
@@ -12164,17 +12159,17 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>ArchiveLifePerLevel</t>
+          <t>EchoesRunWon</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>25</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>STRONGER BAND</t>
+          <t>the whole run won</t>
         </is>
       </c>
     </row>
@@ -12186,17 +12181,17 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>ArchiveBreathPerLevel</t>
+          <t>EchoesMaestro</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>1.5</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>DEEP BREATH</t>
+          <t>MAESTRO pays more</t>
         </is>
       </c>
     </row>
@@ -12208,7 +12203,7 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>ArchiveSignaturePerLevel</t>
+          <t>ArchiveLifePerLevel</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
@@ -12218,7 +12213,7 @@
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>WARM UP</t>
+          <t>STRONGER BAND</t>
         </is>
       </c>
     </row>
@@ -12230,17 +12225,17 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>ArchiveShardsPerLevel</t>
+          <t>ArchiveBreathPerLevel</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>SAVINGS</t>
+          <t>DEEP BREATH</t>
         </is>
       </c>
     </row>
@@ -12252,61 +12247,61 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>ArchiveFirstChairTier</t>
+          <t>ArchiveSignaturePerLevel</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>FIRST CHAIR (29 Oct, was FULL STAGE) : the first musician picked starts with their weapon this many tiers up</t>
+          <t>WARM UP</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>Turn Motifs</t>
+          <t>ARCHIVE</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>TurnReedCaseHeal</t>
+          <t>ArchiveShardsPerLevel</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>1.5</t>
+          <t>20</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>REED CASE : wind players' healing</t>
+          <t>SAVINGS</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>Turn Motifs</t>
+          <t>ARCHIVE</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>TurnSpareSticksOffBeat</t>
+          <t>ArchiveFirstChairTier</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>1.5</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>SPARE STICKS : percussion skills' OFF-BEAT</t>
+          <t>FIRST CHAIR (29 Oct, was FULL STAGE) : the first musician picked starts with their weapon this many tiers up</t>
         </is>
       </c>
     </row>
@@ -12318,17 +12313,17 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>TurnPianissimoBreath</t>
+          <t>TurnReedCaseHeal</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>1.5</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>PIANISSIMO : more breath for the first note of an attack parried PERFECT (was a p note)</t>
+          <t>REED CASE : wind players' healing</t>
         </is>
       </c>
     </row>
@@ -12340,17 +12335,17 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>TurnBreathMarkStart</t>
+          <t>TurnSpareSticksOffBeat</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1.5</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>BREATH MARK : more breath at the start of a fight</t>
+          <t>SPARE STICKS : percussion skills' OFF-BEAT</t>
         </is>
       </c>
     </row>
@@ -12362,17 +12357,17 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>TurnTuttiScale</t>
+          <t>TurnPianissimoBreath</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>1.25</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>TUTTI : skills that reach everyone</t>
+          <t>PIANISSIMO : more breath for the first note of an attack parried PERFECT (was a p note)</t>
         </is>
       </c>
     </row>
@@ -12384,17 +12379,17 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>TurnRubatoMiss</t>
+          <t>TurnBreathMarkStart</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>0.6</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>RUBATO : a skill note you MISS still plays at this (step 12)</t>
+          <t>BREATH MARK : more breath at the start of a fight</t>
         </is>
       </c>
     </row>
@@ -12406,17 +12401,17 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>TurnCrescendoStart</t>
+          <t>TurnTuttiScale</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>1.25</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>CRESCENDO : stacks on every musician at the start</t>
+          <t>TUTTI : skills that reach everyone</t>
         </is>
       </c>
     </row>
@@ -12428,17 +12423,17 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>TurnSforzandoScale</t>
+          <t>TurnRubatoMiss</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>1.3</t>
+          <t>0.6</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>SFORZANDO : the PERFECT last note of a skill (was an f note)</t>
+          <t>RUBATO : a skill note you MISS still plays at this (step 12)</t>
         </is>
       </c>
     </row>
@@ -12450,17 +12445,17 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>TurnOvertureScale</t>
+          <t>TurnCrescendoStart</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>OVERTURE : the band's first hit of a fight</t>
+          <t>CRESCENDO : stacks on every musician at the start</t>
         </is>
       </c>
     </row>
@@ -12472,17 +12467,17 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>TurnCounterpointScale</t>
+          <t>TurnSforzandoScale</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1.3</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
         <is>
-          <t>COUNTERPOINT : the COUNTER</t>
+          <t>SFORZANDO : the PERFECT last note of a skill (was an f note)</t>
         </is>
       </c>
     </row>
@@ -12494,7 +12489,7 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>TurnAccelerandoShakes</t>
+          <t>TurnOvertureScale</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
@@ -12504,7 +12499,7 @@
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>ACCELERANDO : each shake of a roll counts this many</t>
+          <t>OVERTURE : the band's first hit of a fight</t>
         </is>
       </c>
     </row>
@@ -12516,7 +12511,7 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>TurnGraceTimes</t>
+          <t>TurnCounterpointScale</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
@@ -12526,7 +12521,7 @@
       </c>
       <c r="D140" t="inlineStr">
         <is>
-          <t>GRACE NOTE : a spark that lands does its skill this many times</t>
+          <t>COUNTERPOINT : the COUNTER</t>
         </is>
       </c>
     </row>
@@ -12538,7 +12533,7 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>TurnMarcatoOffBeat</t>
+          <t>TurnAccelerandoShakes</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
@@ -12548,7 +12543,7 @@
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>MARCATO : a PERFECT attack's OFF-BEAT, times this</t>
+          <t>ACCELERANDO : each shake of a roll counts this many</t>
         </is>
       </c>
     </row>
@@ -12560,17 +12555,17 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>TurnConBrioNeed</t>
+          <t>TurnGraceTimes</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D142" t="inlineStr">
         <is>
-          <t>CON BRIO : PERFECTs the SIGNATURE needs instead</t>
+          <t>GRACE NOTE : a spark that lands does its skill this many times</t>
         </is>
       </c>
     </row>
@@ -12582,17 +12577,17 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>TurnCodaBelow</t>
+          <t>TurnMarcatoOffBeat</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>0.25</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D143" t="inlineStr">
         <is>
-          <t>CODA : an enemy under this share of its life</t>
+          <t>MARCATO : a PERFECT attack's OFF-BEAT, times this</t>
         </is>
       </c>
     </row>
@@ -12604,61 +12599,61 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>TurnCodaScale</t>
+          <t>TurnConBrioNeed</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>1.5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="D144" t="inlineStr">
         <is>
-          <t>takes this much more</t>
+          <t>CON BRIO : PERFECTs the SIGNATURE needs instead</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>ONE BAR motifs</t>
+          <t>Turn Motifs</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>TurnDownbeatScale</t>
+          <t>TurnCodaBelow</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>1.5</t>
+          <t>0.25</t>
         </is>
       </c>
       <c r="D145" t="inlineStr">
         <is>
-          <t>DOWNBEAT : the first move of a bar</t>
+          <t>CODA : an enemy under this share of its life</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>ONE BAR motifs</t>
+          <t>Turn Motifs</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>TurnEntranceScale</t>
+          <t>TurnCodaScale</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1.5</t>
         </is>
       </c>
       <c r="D146" t="inlineStr">
         <is>
-          <t>ENTRANCE (29 Oct, CALL is gone) : each musician's first move of a fight. Was : a called musician's first bar</t>
+          <t>takes this much more</t>
         </is>
       </c>
     </row>
@@ -12670,17 +12665,17 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>TurnGreenRoomHeal</t>
+          <t>TurnDownbeatScale</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1.5</t>
         </is>
       </c>
       <c r="D147" t="inlineStr">
         <is>
-          <t>GREEN ROOM (29 Oct, the BENCH is gone) : life back for the most hurt musician standing at the end of a</t>
+          <t>DOWNBEAT : the first move of a bar</t>
         </is>
       </c>
     </row>
@@ -12692,7 +12687,7 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>TurnUnisonScale</t>
+          <t>TurnEntranceScale</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
@@ -12702,51 +12697,51 @@
       </c>
       <c r="D148" t="inlineStr">
         <is>
-          <t>UNISON : the last ATTACK of a bar that all goes at one enemy</t>
+          <t>ENTRANCE (29 Oct, CALL is gone) : each musician's first move of a fight. Was : a called musician's first bar</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>Turn Feel</t>
+          <t>ONE BAR motifs</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>TurnRingTime</t>
+          <t>TurnGreenRoomHeal</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>1.1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="D149" t="inlineStr">
         <is>
-          <t>from a note showing to the moment to swipe</t>
+          <t>GREEN ROOM (29 Oct, the BENCH is gone) : life back for the most hurt musician standing at the end of a</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>Turn Feel</t>
+          <t>ONE BAR motifs</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>TurnLateReveal</t>
+          <t>TurnUnisonScale</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>0.5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D150" t="inlineStr">
         <is>
-          <t>FALSE NOTES (STATIC) : its hidden note shows its arrow once the ring is this far closed</t>
+          <t>UNISON : the last ATTACK of a bar that all goes at one enemy</t>
         </is>
       </c>
     </row>
@@ -12758,17 +12753,17 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>MaestroTurnRingTime</t>
+          <t>TurnRingTime</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>0.8</t>
+          <t>1.1</t>
         </is>
       </c>
       <c r="D151" t="inlineStr">
         <is>
-          <t>MAESTRO</t>
+          <t>from a note showing to the moment to swipe</t>
         </is>
       </c>
     </row>
@@ -12780,17 +12775,17 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>TurnNoteGap</t>
+          <t>TurnLateReveal</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>0.55</t>
+          <t>0.5</t>
         </is>
       </c>
       <c r="D152" t="inlineStr">
         <is>
-          <t>between the notes of one enemy attack</t>
+          <t>FALSE NOTES (STATIC) : its hidden note shows its arrow once the ring is this far closed</t>
         </is>
       </c>
     </row>
@@ -12802,7 +12797,7 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>TurnPause</t>
+          <t>MaestroTurnRingTime</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
@@ -12812,7 +12807,7 @@
       </c>
       <c r="D153" t="inlineStr">
         <is>
-          <t>after a turn, before the next one starts</t>
+          <t>MAESTRO</t>
         </is>
       </c>
     </row>
@@ -12824,17 +12819,17 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>TurnHitStop</t>
+          <t>TurnNoteGap</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>0.075</t>
+          <t>0.55</t>
         </is>
       </c>
       <c r="D154" t="inlineStr">
         <is>
-          <t>the band and TACET freeze for a moment on a PERFECT</t>
+          <t>between the notes of one enemy attack</t>
         </is>
       </c>
     </row>
@@ -12846,17 +12841,17 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>TurnStrikeTime</t>
+          <t>TurnPause</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>0.62</t>
+          <t>0.8</t>
         </is>
       </c>
       <c r="D155" t="inlineStr">
         <is>
-          <t>ONE BAR : how long an ATTACK's lunge takes, there and back (Beta1 : slower, smoother)</t>
+          <t>after a turn, before the next one starts</t>
         </is>
       </c>
     </row>
@@ -12868,17 +12863,17 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>TurnStrikeImpact</t>
+          <t>TurnHitStop</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>0.24</t>
+          <t>0.075</t>
         </is>
       </c>
       <c r="D156" t="inlineStr">
         <is>
-          <t>when in it the hit lands</t>
+          <t>the band and TACET freeze for a moment on a PERFECT</t>
         </is>
       </c>
     </row>
@@ -12890,17 +12885,17 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>TurnStrikeStop</t>
+          <t>TurnStrikeTime</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>0.08</t>
+          <t>0.62</t>
         </is>
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t>the freeze when it lands</t>
+          <t>ONE BAR : how long an ATTACK's lunge takes, there and back (Beta1 : slower, smoother)</t>
         </is>
       </c>
     </row>
@@ -12912,17 +12907,17 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>TurnNumberTime</t>
+          <t>TurnStrikeImpact</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>0.24</t>
         </is>
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t>a damage number stays this long (Beta1 round 4, pixel numbers)</t>
+          <t>when in it the hit lands</t>
         </is>
       </c>
     </row>
@@ -12934,17 +12929,17 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>TurnBigHit</t>
+          <t>TurnStrikeStop</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>0.08</t>
         </is>
       </c>
       <c r="D159" t="inlineStr">
         <is>
-          <t>from this much damage it is drawn bigger</t>
+          <t>the freeze when it lands</t>
         </is>
       </c>
     </row>
@@ -12956,17 +12951,17 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>TurnNumberCell</t>
+          <t>TurnNumberTime</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>4.5</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="D160" t="inlineStr">
         <is>
-          <t>one cell of a digit (5 x 7 cells) in pixels (round 4 : 25% smaller, was 6)</t>
+          <t>a damage number stays this long (Beta1 round 4, pixel numbers)</t>
         </is>
       </c>
     </row>
@@ -12978,17 +12973,17 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>TurnNumberBigCell</t>
+          <t>TurnBigHit</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>18</t>
         </is>
       </c>
       <c r="D161" t="inlineStr">
         <is>
-          <t>the same for a big hit (was 8)</t>
+          <t>from this much damage it is drawn bigger</t>
         </is>
       </c>
     </row>
@@ -13000,17 +12995,17 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>TurnDissolveTime</t>
+          <t>TurnNumberCell</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>4.5</t>
         </is>
       </c>
       <c r="D162" t="inlineStr">
         <is>
-          <t>an enemy SILENCED dissolves into TACET's hole in this long</t>
+          <t>one cell of a digit (5 x 7 cells) in pixels (round 4 : 25% smaller, was 6)</t>
         </is>
       </c>
     </row>
@@ -13022,17 +13017,17 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>TurnCutInTime</t>
+          <t>TurnNumberBigCell</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>1.3</t>
+          <t>6</t>
         </is>
       </c>
       <c r="D163" t="inlineStr">
         <is>
-          <t>the SIGNATURE's CUT-IN, before its strokes (Beta1 round 4, the old duel's picture)</t>
+          <t>the same for a big hit (was 8)</t>
         </is>
       </c>
     </row>
@@ -13044,17 +13039,17 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>TurnKillStop</t>
+          <t>TurnDissolveTime</t>
         </is>
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>0.18</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="D164" t="inlineStr">
         <is>
-          <t>the freeze when an enemy falls silent</t>
+          <t>an enemy SILENCED dissolves into TACET's hole in this long</t>
         </is>
       </c>
     </row>
@@ -13066,17 +13061,17 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>TurnEndTime</t>
+          <t>TurnCutInTime</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>2.2</t>
+          <t>1.3</t>
         </is>
       </c>
       <c r="D165" t="inlineStr">
         <is>
-          <t>the win or lose banner stays this long</t>
+          <t>the SIGNATURE's CUT-IN, before its strokes (Beta1 round 4, the old duel's picture)</t>
         </is>
       </c>
     </row>
@@ -13088,17 +13083,17 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>TurnSparkGap</t>
+          <t>TurnKillStop</t>
         </is>
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>0.3</t>
+          <t>0.18</t>
         </is>
       </c>
       <c r="D166" t="inlineStr">
         <is>
-          <t>a spark comes this soon after the note before it</t>
+          <t>the freeze when an enemy falls silent</t>
         </is>
       </c>
     </row>
@@ -13110,17 +13105,17 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>TurnHoldTime</t>
+          <t>TurnEndTime</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>0.8</t>
+          <t>2.2</t>
         </is>
       </c>
       <c r="D167" t="inlineStr">
         <is>
-          <t>how long a HOLD note wants holding (the button kept down, the baton may move : Beta1 29 Oct)</t>
+          <t>the win or lose banner stays this long</t>
         </is>
       </c>
     </row>
@@ -13132,15 +13127,59 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
+          <t>TurnSparkGap</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>0.3</t>
+        </is>
+      </c>
+      <c r="D168" t="inlineStr">
+        <is>
+          <t>a spark comes this soon after the note before it</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>Turn Feel</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>TurnHoldTime</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>0.8</t>
+        </is>
+      </c>
+      <c r="D169" t="inlineStr">
+        <is>
+          <t>how long a HOLD note wants holding (the button kept down, the baton may move : Beta1 29 Oct)</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>Turn Feel</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
           <t>TurnRollTime</t>
         </is>
       </c>
-      <c r="C168" t="inlineStr">
+      <c r="C170" t="inlineStr">
         <is>
           <t>1.2</t>
         </is>
       </c>
-      <c r="D168" t="inlineStr">
+      <c r="D170" t="inlineStr">
         <is>
           <t>how long a ROLL note lasts</t>
         </is>

</xml_diff>